<commit_message>
Sprint Backlogs S2–S5 marcados con lo hecho por Bryan; MD 10.9
S4: 81 tareas terminadas, 10 bloqueadas por desarrollos de otros; 12
historias en revisión; 30 criterios verificados. S3: HU-076 tomada y
terminada, T-3261 desbloqueada, decisión HU-073 #3. S5: HU-111 reasignada
a Bryan y terminada. S2: HU-041 tomada y terminada.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S2.xlsx
+++ b/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" tabRatio="500" firstSheet="1" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sprint" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Historias" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Tareas" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Criterios de aceptación" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Definition of Done" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historias" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tareas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Criterios de aceptación" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Definition of Done" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Historias'!$A$5:$P$27</definedName>
@@ -1149,8 +1149,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="27.75" customHeight="1" s="19">
       <c r="A5" s="10" t="inlineStr">
         <is>
@@ -2521,11 +2519,19 @@
       </c>
       <c r="N23" s="13" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="O23" s="14" t="n"/>
-      <c r="P23" s="14" t="n"/>
+          <t>En revisión</t>
+        </is>
+      </c>
+      <c r="O23" s="14" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
+      <c r="P23" s="14" t="inlineStr">
+        <is>
+          <t>Tomada por Bryan el 12-09-2026 porque bloqueaba HU-074 (S3). Hecha y verificada.</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="69" customHeight="1" s="19">
       <c r="A24" s="11" t="inlineStr">
@@ -11457,11 +11463,17 @@
       </c>
       <c r="H202" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I202" s="11" t="n"/>
-      <c r="J202" s="12" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I202" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J202" s="12" t="inlineStr">
+        <is>
+          <t>BD/224. Sin código: única por (equipo, componente, variable). CK min&lt;=max en tabla; el orden completo de umbrales en el SP.</t>
+        </is>
+      </c>
     </row>
     <row r="203" hidden="1" ht="27.6" customHeight="1" s="19">
       <c r="A203" s="11" t="inlineStr">
@@ -11494,16 +11506,22 @@
       </c>
       <c r="G203" s="12" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H203" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I203" s="11" t="n"/>
-      <c r="J203" s="12" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I203" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J203" s="12" t="inlineStr">
+        <is>
+          <t>SEL completo (reemplaza el mínimo del bloque 105; conserva ETIQUETA para el combo de condiciones).</t>
+        </is>
+      </c>
     </row>
     <row r="204" hidden="1" ht="41.4" customHeight="1" s="19">
       <c r="A204" s="11" t="inlineStr">
@@ -11536,16 +11554,22 @@
       </c>
       <c r="G204" s="12" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H204" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I204" s="11" t="n"/>
-      <c r="J204" s="12" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I204" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J204" s="12" t="inlineStr">
+        <is>
+          <t>INS: equipo del cliente, componente del equipo, variable habilitada, unidad por defecto la de la variable, terna única.</t>
+        </is>
+      </c>
     </row>
     <row r="205" hidden="1" ht="27.6" customHeight="1" s="19">
       <c r="A205" s="11" t="inlineStr">
@@ -11583,11 +11607,17 @@
       </c>
       <c r="H205" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I205" s="11" t="n"/>
-      <c r="J205" s="12" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I205" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J205" s="12" t="inlineStr">
+        <is>
+          <t>UPD con QUITA_* para vaciar umbrales; equipo/variable no cambian.</t>
+        </is>
+      </c>
     </row>
     <row r="206" hidden="1" ht="27.6" customHeight="1" s="19">
       <c r="A206" s="11" t="inlineStr">
@@ -11620,16 +11650,22 @@
       </c>
       <c r="G206" s="12" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H206" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I206" s="11" t="n"/>
-      <c r="J206" s="12" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I206" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J206" s="12" t="inlineStr">
+        <is>
+          <t>DEL lógico; rechaza si una programación por condición vigila la variable.</t>
+        </is>
+      </c>
     </row>
     <row r="207" hidden="1" ht="27.6" customHeight="1" s="19">
       <c r="A207" s="11" t="inlineStr">
@@ -11662,16 +11698,22 @@
       </c>
       <c r="G207" s="12" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H207" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I207" s="11" t="n"/>
-      <c r="J207" s="12" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I207" s="11" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J207" s="12" t="inlineStr">
+        <is>
+          <t>Ya había 9 filas descubiertas por la app (HU-155); se creó ACT-41 · Vibración desde la web.</t>
+        </is>
+      </c>
     </row>
     <row r="208" hidden="1" ht="27.6" customHeight="1" s="19">
       <c r="A208" s="11" t="inlineStr">
@@ -11704,16 +11746,22 @@
       </c>
       <c r="G208" s="12" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H208" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I208" s="11" t="n"/>
-      <c r="J208" s="12" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I208" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J208" s="12" t="inlineStr">
+        <is>
+          <t>View/Activos/Variables/ActivoVariables.aspx con umbrales como chips y filtro por planta.</t>
+        </is>
+      </c>
     </row>
     <row r="209" hidden="1" ht="27.6" customHeight="1" s="19">
       <c r="A209" s="11" t="inlineStr">
@@ -11751,11 +11799,17 @@
       </c>
       <c r="H209" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I209" s="11" t="n"/>
-      <c r="J209" s="12" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I209" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J209" s="12" t="inlineStr">
+        <is>
+          <t>ActivoVariable.aspx: equipo→componente en cascada; umbrales fuera de orden y variable repetida rechazados con mensaje (verificado).</t>
+        </is>
+      </c>
     </row>
     <row r="210" hidden="1" ht="55.2" customHeight="1" s="19">
       <c r="A210" s="11" t="inlineStr">
@@ -11788,16 +11842,22 @@
       </c>
       <c r="G210" s="12" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H210" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I210" s="11" t="n"/>
-      <c r="J210" s="12" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I210" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J210" s="12" t="inlineStr">
+        <is>
+          <t>Menús «Variables de condición» (visible) y detalle (99) junto a Medidores; Menu_Funcion.</t>
+        </is>
+      </c>
     </row>
     <row r="211" hidden="1" ht="41.4" customHeight="1" s="19">
       <c r="A211" s="11" t="inlineStr">
@@ -11830,16 +11890,22 @@
       </c>
       <c r="G211" s="12" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H211" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I211" s="11" t="n"/>
-      <c r="J211" s="12" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I211" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J211" s="12" t="inlineStr">
+        <is>
+          <t>Permisos VER/CREAR EDITAR VARIABLES ACTIVO a los perfiles de medidores; cliente desde la sesión.</t>
+        </is>
+      </c>
     </row>
     <row r="212" hidden="1" ht="41.4" customHeight="1" s="19">
       <c r="A212" s="11" t="inlineStr">
@@ -11872,16 +11938,22 @@
       </c>
       <c r="G212" s="12" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H212" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I212" s="11" t="n"/>
-      <c r="J212" s="12" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I212" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J212" s="12" t="inlineStr">
+        <is>
+          <t>Criterio 1 (alta con unidad) verificado; criterio 2 (mediciones validadas contra umbrales) lo hace la app al registrar medición (HU-044).</t>
+        </is>
+      </c>
     </row>
     <row r="213" hidden="1" ht="41.4" customHeight="1" s="19">
       <c r="A213" s="11" t="inlineStr">
@@ -11914,16 +11986,22 @@
       </c>
       <c r="G213" s="12" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H213" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I213" s="11" t="n"/>
-      <c r="J213" s="12" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I213" s="11" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J213" s="12" t="inlineStr">
+        <is>
+          <t>MD 10.9.</t>
+        </is>
+      </c>
     </row>
     <row r="214" hidden="1" ht="41.4" customHeight="1" s="19">
       <c r="A214" s="11" t="inlineStr">
@@ -15479,7 +15557,7 @@
       </c>
       <c r="F53" s="13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sprint 2: captura en terreno completa (HU-043, HU-044, HU-038)
- App: CapturaScreen encolaba el cuerpo con nombres que la API no conoce
  (act_id, ame_id, fecha_evento) y la medicion no llevaba variable: cada
  captura rebotaba. Ahora usa los nombres del DTO con uuid, la ficha del
  activo pide elegir la variable (sabana MEDICION_1) y exige comentario
  fuera de umbral; la lectura se registra desde el medidor.
- BD/235: ame_maximo_diario y salto no razonable -> lectura pendiente de
  revision + alerta LECTURA A REVISAR (HU-043 #2); veredicto sobre el
  equivalente en la unidad de la variable (HU-044 #1); comentario
  obligatorio y alerta MEDICION FUERA RANGO (HU-044 #2); origen ORDEN
  TRABAJO en lecturas y mediciones con OT.
- Web: campo "Maximo diario" en la ficha del medidor.
- API: POST /captura/lecturas devuelve {id, mensaje}.
- Evidencia S2 (41 casos, 40 ok); todas las tareas de Bryan del S2 cerradas.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S2.xlsx
+++ b/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Capstone\SIGMA\Fase 2\Sprint Backlogs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BD2684E-BCA6-438D-97A3-72E98A3F7FC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FE97F4A-C77F-497E-A0F0-76524D122FAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2493" uniqueCount="833">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2504" uniqueCount="844">
   <si>
     <t>Sprint 2 · Historias comprometidas</t>
   </si>
@@ -974,6 +974,9 @@
     <t>SP INS_ACTIVO_MEDIDOR_LECTURA: alta transaccional con las validaciones de negocio de la historia. Devuelve el id creado por OUTPUT.</t>
   </si>
   <si>
+    <t>API_INS_ACTIVO_MEDIDOR_LECTURA (141) + salto no razonable → pendiente de revisión y alerta (BD/235)</t>
+  </si>
+  <si>
     <t>T-2062</t>
   </si>
   <si>
@@ -992,6 +995,9 @@
     <t>Datos de prueba en Activo_Medidor_Lectura para poder ejercitar los criterios de aceptación.</t>
   </si>
   <si>
+    <t>MED-33-H con máximo diario 24 h; lecturas de ronda y salto de 400 h</t>
+  </si>
+  <si>
     <t>T-2065</t>
   </si>
   <si>
@@ -1004,6 +1010,9 @@
     <t>GET /api/activo-medidor-lecturas/{id} y GET /api/activo-medidor-lecturas — detalle y listado.</t>
   </si>
   <si>
+    <t>GET /medidores/{id} y GET /medidores/{id}/lecturas (bloque 203)</t>
+  </si>
+  <si>
     <t>T-2067</t>
   </si>
   <si>
@@ -1013,9 +1022,15 @@
     <t>T-2070</t>
   </si>
   <si>
+    <t>CapturaScreen desde el medidor; cuerpo con los nombres del DTO (defecto corregido 16-09)</t>
+  </si>
+  <si>
     <t>T-2071</t>
   </si>
   <si>
+    <t>REGISTRAR LECTURA en la API; medidor validado contra el cliente del token</t>
+  </si>
+  <si>
     <t>T-2072</t>
   </si>
   <si>
@@ -1232,6 +1247,9 @@
     <t>SP INS_ACTIVO_MEDICION: alta transaccional con las validaciones de negocio de la historia. Devuelve el id creado por OUTPUT.</t>
   </si>
   <si>
+    <t>API_INS_ACTIVO_MEDICION: equivalente en la unidad de la variable, comentario obligatorio fuera de umbral y alerta (BD/235)</t>
+  </si>
+  <si>
     <t>T-2122</t>
   </si>
   <si>
@@ -1250,6 +1268,9 @@
     <t>Datos de prueba en Activo_Medicion para poder ejercitar los criterios de aceptación.</t>
   </si>
   <si>
+    <t>Variable Presión en bar de ACT-36; mediciones en psi y bar</t>
+  </si>
+  <si>
     <t>T-2125</t>
   </si>
   <si>
@@ -1262,15 +1283,24 @@
     <t>GET /api/activo-mediciones/{id} y GET /api/activo-mediciones — detalle y listado.</t>
   </si>
   <si>
+    <t>GET /captura/mediciones se cubre con la serie web (BD/233); detalle por Alerta</t>
+  </si>
+  <si>
     <t>T-2127</t>
   </si>
   <si>
     <t>T-2130</t>
   </si>
   <si>
+    <t>CapturaScreen elige la variable (sábana) y pide comentario fuera de umbral</t>
+  </si>
+  <si>
     <t>T-2131</t>
   </si>
   <si>
+    <t>REGISTRAR MEDICION en la API; variable validada contra el cliente del token</t>
+  </si>
+  <si>
     <t>T-2132</t>
   </si>
   <si>
@@ -1409,6 +1439,9 @@
     <t>T-2154</t>
   </si>
   <si>
+    <t>POST /activo-estados con motivo obligatorio y cierre del periodo anterior (evidencia HU-038)</t>
+  </si>
+  <si>
     <t>T-2155</t>
   </si>
   <si>
@@ -1703,7 +1736,7 @@
     <t>Datos de prueba en Suscripcion_Pago para poder ejercitar los criterios de aceptación.</t>
   </si>
   <si>
-    <t>PENDIENTE al 02-09-2026: Suscripcion_Pago tiene 0 filas. Sin un pago cargado no hay como ejercitar los criterios de la historia. · Script de siembra escrito y ejecutado (bloque 59 §3), pero NO sembró: Suscripcion_Periodo tiene 0 filas. No crea la suscripción a propósito -el 29-08 se pidió expresamente crearla desde la web-. Es idempotente: cree la suscripción y emita un período desde la web, y vuelva a ejecutar SOLO la sección 3 del bloque 59. Siembra 3 pagos: uno declarado, uno rechazado para corregir, y uno parcial.</t>
+    <t>Suscripcion_Pago con pagos declarados, rechazados y verificados (evidencia HU-194)</t>
   </si>
   <si>
     <t>T-2216</t>
@@ -6568,14 +6601,18 @@
         <v>85</v>
       </c>
       <c r="H57" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="I57" s="11"/>
-      <c r="J57" s="12"/>
+        <v>137</v>
+      </c>
+      <c r="I57" s="11">
+        <v>0.5</v>
+      </c>
+      <c r="J57" s="12" t="s">
+        <v>309</v>
+      </c>
     </row>
     <row r="58" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B58" s="11" t="s">
         <v>52</v>
@@ -6584,7 +6621,7 @@
         <v>53</v>
       </c>
       <c r="D58" s="17" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E58" s="11" t="s">
         <v>199</v>
@@ -6603,7 +6640,7 @@
     </row>
     <row r="59" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="11" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B59" s="11" t="s">
         <v>52</v>
@@ -6612,7 +6649,7 @@
         <v>53</v>
       </c>
       <c r="D59" s="17" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E59" s="11" t="s">
         <v>199</v>
@@ -6631,7 +6668,7 @@
     </row>
     <row r="60" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="11" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B60" s="11" t="s">
         <v>52</v>
@@ -6640,7 +6677,7 @@
         <v>53</v>
       </c>
       <c r="D60" s="17" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E60" s="11" t="s">
         <v>199</v>
@@ -6652,14 +6689,18 @@
         <v>85</v>
       </c>
       <c r="H60" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="I60" s="11"/>
-      <c r="J60" s="12"/>
+        <v>137</v>
+      </c>
+      <c r="I60" s="11">
+        <v>0.25</v>
+      </c>
+      <c r="J60" s="12" t="s">
+        <v>316</v>
+      </c>
     </row>
     <row r="61" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="11" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B61" s="11" t="s">
         <v>52</v>
@@ -6668,7 +6709,7 @@
         <v>53</v>
       </c>
       <c r="D61" s="17" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="E61" s="11" t="s">
         <v>263</v>
@@ -6687,7 +6728,7 @@
     </row>
     <row r="62" spans="1:10" ht="55.15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="11" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B62" s="11" t="s">
         <v>52</v>
@@ -6696,7 +6737,7 @@
         <v>53</v>
       </c>
       <c r="D62" s="17" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="E62" s="11" t="s">
         <v>263</v>
@@ -6708,14 +6749,18 @@
         <v>85</v>
       </c>
       <c r="H62" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="I62" s="11"/>
-      <c r="J62" s="12"/>
+        <v>137</v>
+      </c>
+      <c r="I62" s="11">
+        <v>0.25</v>
+      </c>
+      <c r="J62" s="12" t="s">
+        <v>321</v>
+      </c>
     </row>
     <row r="63" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="11" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="B63" s="11" t="s">
         <v>52</v>
@@ -6724,7 +6769,7 @@
         <v>53</v>
       </c>
       <c r="D63" s="17" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="E63" s="11" t="s">
         <v>263</v>
@@ -6743,7 +6788,7 @@
     </row>
     <row r="64" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="11" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="B64" s="11" t="s">
         <v>52</v>
@@ -6764,14 +6809,18 @@
         <v>85</v>
       </c>
       <c r="H64" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="I64" s="11"/>
-      <c r="J64" s="12"/>
+        <v>137</v>
+      </c>
+      <c r="I64" s="11">
+        <v>0.25</v>
+      </c>
+      <c r="J64" s="12" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="65" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="11" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="B65" s="11" t="s">
         <v>52</v>
@@ -6792,14 +6841,18 @@
         <v>85</v>
       </c>
       <c r="H65" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="I65" s="11"/>
-      <c r="J65" s="12"/>
+        <v>137</v>
+      </c>
+      <c r="I65" s="11">
+        <v>0.25</v>
+      </c>
+      <c r="J65" s="12" t="s">
+        <v>327</v>
+      </c>
     </row>
     <row r="66" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="11" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="B66" s="11" t="s">
         <v>52</v>
@@ -6827,7 +6880,7 @@
     </row>
     <row r="67" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="11" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="B67" s="11" t="s">
         <v>52</v>
@@ -6855,7 +6908,7 @@
     </row>
     <row r="68" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="11" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="B68" s="11" t="s">
         <v>57</v>
@@ -6864,7 +6917,7 @@
         <v>58</v>
       </c>
       <c r="D68" s="17" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="E68" s="11" t="s">
         <v>199</v>
@@ -6883,7 +6936,7 @@
     </row>
     <row r="69" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="11" t="s">
-        <v>327</v>
+        <v>332</v>
       </c>
       <c r="B69" s="11" t="s">
         <v>57</v>
@@ -6892,7 +6945,7 @@
         <v>58</v>
       </c>
       <c r="D69" s="17" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="E69" s="11" t="s">
         <v>199</v>
@@ -6911,7 +6964,7 @@
     </row>
     <row r="70" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="11" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="B70" s="11" t="s">
         <v>57</v>
@@ -6920,7 +6973,7 @@
         <v>58</v>
       </c>
       <c r="D70" s="17" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="E70" s="11" t="s">
         <v>199</v>
@@ -6938,12 +6991,12 @@
         <v>0.5</v>
       </c>
       <c r="J70" s="12" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
     </row>
     <row r="71" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="11" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="B71" s="11" t="s">
         <v>57</v>
@@ -6952,7 +7005,7 @@
         <v>58</v>
       </c>
       <c r="D71" s="17" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="E71" s="11" t="s">
         <v>199</v>
@@ -6971,7 +7024,7 @@
     </row>
     <row r="72" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="11" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="B72" s="11" t="s">
         <v>57</v>
@@ -6980,7 +7033,7 @@
         <v>58</v>
       </c>
       <c r="D72" s="17" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="E72" s="11" t="s">
         <v>263</v>
@@ -6998,12 +7051,12 @@
         <v>0.75</v>
       </c>
       <c r="J72" s="12" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
     </row>
     <row r="73" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="11" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
       <c r="B73" s="11" t="s">
         <v>57</v>
@@ -7012,7 +7065,7 @@
         <v>58</v>
       </c>
       <c r="D73" s="17" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
       <c r="E73" s="11" t="s">
         <v>263</v>
@@ -7031,7 +7084,7 @@
     </row>
     <row r="74" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="11" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="B74" s="11" t="s">
         <v>57</v>
@@ -7058,12 +7111,12 @@
         <v>0.5</v>
       </c>
       <c r="J74" s="12" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
     </row>
     <row r="75" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="11" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="B75" s="11" t="s">
         <v>57</v>
@@ -7072,7 +7125,7 @@
         <v>58</v>
       </c>
       <c r="D75" s="17" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="E75" s="11" t="s">
         <v>273</v>
@@ -7091,7 +7144,7 @@
     </row>
     <row r="76" spans="1:10" ht="55.15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="11" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
       <c r="B76" s="11" t="s">
         <v>57</v>
@@ -7118,12 +7171,12 @@
         <v>0.25</v>
       </c>
       <c r="J76" s="12" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
     </row>
     <row r="77" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="11" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="B77" s="11" t="s">
         <v>57</v>
@@ -7151,7 +7204,7 @@
     </row>
     <row r="78" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="11" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="B78" s="11" t="s">
         <v>57</v>
@@ -7179,7 +7232,7 @@
     </row>
     <row r="79" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="11" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="B79" s="11" t="s">
         <v>57</v>
@@ -7207,7 +7260,7 @@
     </row>
     <row r="80" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="11" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="B80" s="11" t="s">
         <v>57</v>
@@ -7235,7 +7288,7 @@
     </row>
     <row r="81" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="11" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
       <c r="B81" s="11" t="s">
         <v>62</v>
@@ -7244,7 +7297,7 @@
         <v>63</v>
       </c>
       <c r="D81" s="17" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="E81" s="11" t="s">
         <v>199</v>
@@ -7263,7 +7316,7 @@
     </row>
     <row r="82" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="11" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="B82" s="11" t="s">
         <v>62</v>
@@ -7272,7 +7325,7 @@
         <v>63</v>
       </c>
       <c r="D82" s="17" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
       <c r="E82" s="11" t="s">
         <v>199</v>
@@ -7290,12 +7343,12 @@
         <v>0.5</v>
       </c>
       <c r="J82" s="12" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
     </row>
     <row r="83" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="11" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
       <c r="B83" s="11" t="s">
         <v>62</v>
@@ -7304,7 +7357,7 @@
         <v>63</v>
       </c>
       <c r="D83" s="17" t="s">
-        <v>354</v>
+        <v>359</v>
       </c>
       <c r="E83" s="11" t="s">
         <v>199</v>
@@ -7323,7 +7376,7 @@
     </row>
     <row r="84" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="11" t="s">
-        <v>355</v>
+        <v>360</v>
       </c>
       <c r="B84" s="11" t="s">
         <v>62</v>
@@ -7332,7 +7385,7 @@
         <v>63</v>
       </c>
       <c r="D84" s="17" t="s">
-        <v>356</v>
+        <v>361</v>
       </c>
       <c r="E84" s="11" t="s">
         <v>199</v>
@@ -7351,7 +7404,7 @@
     </row>
     <row r="85" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="11" t="s">
-        <v>357</v>
+        <v>362</v>
       </c>
       <c r="B85" s="11" t="s">
         <v>62</v>
@@ -7360,7 +7413,7 @@
         <v>63</v>
       </c>
       <c r="D85" s="17" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="E85" s="11" t="s">
         <v>199</v>
@@ -7378,12 +7431,12 @@
         <v>0.5</v>
       </c>
       <c r="J85" s="12" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
     </row>
     <row r="86" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="11" t="s">
-        <v>360</v>
+        <v>365</v>
       </c>
       <c r="B86" s="11" t="s">
         <v>62</v>
@@ -7392,7 +7445,7 @@
         <v>63</v>
       </c>
       <c r="D86" s="17" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="E86" s="11" t="s">
         <v>199</v>
@@ -7411,7 +7464,7 @@
     </row>
     <row r="87" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="11" t="s">
-        <v>361</v>
+        <v>366</v>
       </c>
       <c r="B87" s="11" t="s">
         <v>62</v>
@@ -7420,7 +7473,7 @@
         <v>63</v>
       </c>
       <c r="D87" s="17" t="s">
-        <v>362</v>
+        <v>367</v>
       </c>
       <c r="E87" s="11" t="s">
         <v>24</v>
@@ -7439,7 +7492,7 @@
     </row>
     <row r="88" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="11" t="s">
-        <v>363</v>
+        <v>368</v>
       </c>
       <c r="B88" s="11" t="s">
         <v>62</v>
@@ -7448,7 +7501,7 @@
         <v>63</v>
       </c>
       <c r="D88" s="17" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="E88" s="11" t="s">
         <v>24</v>
@@ -7466,12 +7519,12 @@
         <v>0.5</v>
       </c>
       <c r="J88" s="12" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
     </row>
     <row r="89" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="11" t="s">
-        <v>366</v>
+        <v>371</v>
       </c>
       <c r="B89" s="11" t="s">
         <v>62</v>
@@ -7499,7 +7552,7 @@
     </row>
     <row r="90" spans="1:10" ht="55.15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="11" t="s">
-        <v>367</v>
+        <v>372</v>
       </c>
       <c r="B90" s="11" t="s">
         <v>62</v>
@@ -7526,12 +7579,12 @@
         <v>0.5</v>
       </c>
       <c r="J90" s="12" t="s">
-        <v>368</v>
+        <v>373</v>
       </c>
     </row>
     <row r="91" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="11" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="B91" s="11" t="s">
         <v>62</v>
@@ -7559,7 +7612,7 @@
     </row>
     <row r="92" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="11" t="s">
-        <v>370</v>
+        <v>375</v>
       </c>
       <c r="B92" s="11" t="s">
         <v>62</v>
@@ -7587,7 +7640,7 @@
     </row>
     <row r="93" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="11" t="s">
-        <v>371</v>
+        <v>376</v>
       </c>
       <c r="B93" s="11" t="s">
         <v>67</v>
@@ -7596,7 +7649,7 @@
         <v>68</v>
       </c>
       <c r="D93" s="17" t="s">
-        <v>372</v>
+        <v>377</v>
       </c>
       <c r="E93" s="11" t="s">
         <v>199</v>
@@ -7615,7 +7668,7 @@
     </row>
     <row r="94" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="11" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="B94" s="11" t="s">
         <v>67</v>
@@ -7624,7 +7677,7 @@
         <v>68</v>
       </c>
       <c r="D94" s="17" t="s">
-        <v>374</v>
+        <v>379</v>
       </c>
       <c r="E94" s="11" t="s">
         <v>199</v>
@@ -7643,7 +7696,7 @@
     </row>
     <row r="95" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="11" t="s">
-        <v>375</v>
+        <v>380</v>
       </c>
       <c r="B95" s="11" t="s">
         <v>67</v>
@@ -7652,7 +7705,7 @@
         <v>68</v>
       </c>
       <c r="D95" s="17" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="E95" s="11" t="s">
         <v>199</v>
@@ -7671,7 +7724,7 @@
     </row>
     <row r="96" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="11" t="s">
-        <v>377</v>
+        <v>382</v>
       </c>
       <c r="B96" s="11" t="s">
         <v>67</v>
@@ -7680,7 +7733,7 @@
         <v>68</v>
       </c>
       <c r="D96" s="17" t="s">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="E96" s="11" t="s">
         <v>199</v>
@@ -7699,7 +7752,7 @@
     </row>
     <row r="97" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="11" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
       <c r="B97" s="11" t="s">
         <v>67</v>
@@ -7708,7 +7761,7 @@
         <v>68</v>
       </c>
       <c r="D97" s="17" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="E97" s="11" t="s">
         <v>199</v>
@@ -7727,7 +7780,7 @@
     </row>
     <row r="98" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="11" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="B98" s="11" t="s">
         <v>67</v>
@@ -7736,7 +7789,7 @@
         <v>68</v>
       </c>
       <c r="D98" s="17" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="E98" s="11" t="s">
         <v>199</v>
@@ -7755,7 +7808,7 @@
     </row>
     <row r="99" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="11" t="s">
-        <v>383</v>
+        <v>388</v>
       </c>
       <c r="B99" s="11" t="s">
         <v>67</v>
@@ -7764,7 +7817,7 @@
         <v>68</v>
       </c>
       <c r="D99" s="17" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="E99" s="11" t="s">
         <v>24</v>
@@ -7783,7 +7836,7 @@
     </row>
     <row r="100" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="11" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="B100" s="11" t="s">
         <v>67</v>
@@ -7792,7 +7845,7 @@
         <v>68</v>
       </c>
       <c r="D100" s="17" t="s">
-        <v>386</v>
+        <v>391</v>
       </c>
       <c r="E100" s="11" t="s">
         <v>24</v>
@@ -7811,7 +7864,7 @@
     </row>
     <row r="101" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="11" t="s">
-        <v>387</v>
+        <v>392</v>
       </c>
       <c r="B101" s="11" t="s">
         <v>67</v>
@@ -7839,7 +7892,7 @@
     </row>
     <row r="102" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="11" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
       <c r="B102" s="11" t="s">
         <v>67</v>
@@ -7867,7 +7920,7 @@
     </row>
     <row r="103" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="11" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="B103" s="11" t="s">
         <v>67</v>
@@ -7895,7 +7948,7 @@
     </row>
     <row r="104" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="11" t="s">
-        <v>390</v>
+        <v>395</v>
       </c>
       <c r="B104" s="11" t="s">
         <v>67</v>
@@ -7923,7 +7976,7 @@
     </row>
     <row r="105" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="11" t="s">
-        <v>391</v>
+        <v>396</v>
       </c>
       <c r="B105" s="11" t="s">
         <v>73</v>
@@ -7932,7 +7985,7 @@
         <v>74</v>
       </c>
       <c r="D105" s="17" t="s">
-        <v>392</v>
+        <v>397</v>
       </c>
       <c r="E105" s="11" t="s">
         <v>199</v>
@@ -7951,7 +8004,7 @@
     </row>
     <row r="106" spans="1:10" ht="55.15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="11" t="s">
-        <v>393</v>
+        <v>398</v>
       </c>
       <c r="B106" s="11" t="s">
         <v>73</v>
@@ -7960,7 +8013,7 @@
         <v>74</v>
       </c>
       <c r="D106" s="17" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="E106" s="11" t="s">
         <v>199</v>
@@ -7972,14 +8025,18 @@
         <v>85</v>
       </c>
       <c r="H106" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="I106" s="11"/>
-      <c r="J106" s="12"/>
+        <v>137</v>
+      </c>
+      <c r="I106" s="11">
+        <v>0.5</v>
+      </c>
+      <c r="J106" s="12" t="s">
+        <v>400</v>
+      </c>
     </row>
     <row r="107" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="11" t="s">
-        <v>395</v>
+        <v>401</v>
       </c>
       <c r="B107" s="11" t="s">
         <v>73</v>
@@ -7988,7 +8045,7 @@
         <v>74</v>
       </c>
       <c r="D107" s="17" t="s">
-        <v>396</v>
+        <v>402</v>
       </c>
       <c r="E107" s="11" t="s">
         <v>199</v>
@@ -8007,7 +8064,7 @@
     </row>
     <row r="108" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="11" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
       <c r="B108" s="11" t="s">
         <v>73</v>
@@ -8016,7 +8073,7 @@
         <v>74</v>
       </c>
       <c r="D108" s="17" t="s">
-        <v>398</v>
+        <v>404</v>
       </c>
       <c r="E108" s="11" t="s">
         <v>199</v>
@@ -8035,7 +8092,7 @@
     </row>
     <row r="109" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="11" t="s">
-        <v>399</v>
+        <v>405</v>
       </c>
       <c r="B109" s="11" t="s">
         <v>73</v>
@@ -8044,7 +8101,7 @@
         <v>74</v>
       </c>
       <c r="D109" s="17" t="s">
-        <v>400</v>
+        <v>406</v>
       </c>
       <c r="E109" s="11" t="s">
         <v>199</v>
@@ -8056,14 +8113,18 @@
         <v>85</v>
       </c>
       <c r="H109" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="I109" s="11"/>
-      <c r="J109" s="12"/>
+        <v>137</v>
+      </c>
+      <c r="I109" s="11">
+        <v>0.5</v>
+      </c>
+      <c r="J109" s="12" t="s">
+        <v>407</v>
+      </c>
     </row>
     <row r="110" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="11" t="s">
-        <v>401</v>
+        <v>408</v>
       </c>
       <c r="B110" s="11" t="s">
         <v>73</v>
@@ -8072,7 +8133,7 @@
         <v>74</v>
       </c>
       <c r="D110" s="17" t="s">
-        <v>402</v>
+        <v>409</v>
       </c>
       <c r="E110" s="11" t="s">
         <v>263</v>
@@ -8091,7 +8152,7 @@
     </row>
     <row r="111" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="11" t="s">
-        <v>403</v>
+        <v>410</v>
       </c>
       <c r="B111" s="11" t="s">
         <v>73</v>
@@ -8100,7 +8161,7 @@
         <v>74</v>
       </c>
       <c r="D111" s="17" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="E111" s="11" t="s">
         <v>263</v>
@@ -8112,14 +8173,18 @@
         <v>85</v>
       </c>
       <c r="H111" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="I111" s="11"/>
-      <c r="J111" s="12"/>
+        <v>137</v>
+      </c>
+      <c r="I111" s="11">
+        <v>0.5</v>
+      </c>
+      <c r="J111" s="12" t="s">
+        <v>412</v>
+      </c>
     </row>
     <row r="112" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="11" t="s">
-        <v>405</v>
+        <v>413</v>
       </c>
       <c r="B112" s="11" t="s">
         <v>73</v>
@@ -8128,7 +8193,7 @@
         <v>74</v>
       </c>
       <c r="D112" s="17" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="E112" s="11" t="s">
         <v>263</v>
@@ -8147,7 +8212,7 @@
     </row>
     <row r="113" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="11" t="s">
-        <v>406</v>
+        <v>414</v>
       </c>
       <c r="B113" s="11" t="s">
         <v>73</v>
@@ -8168,14 +8233,18 @@
         <v>85</v>
       </c>
       <c r="H113" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="I113" s="11"/>
-      <c r="J113" s="12"/>
+        <v>137</v>
+      </c>
+      <c r="I113" s="11">
+        <v>0.5</v>
+      </c>
+      <c r="J113" s="12" t="s">
+        <v>415</v>
+      </c>
     </row>
     <row r="114" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A114" s="11" t="s">
-        <v>407</v>
+        <v>416</v>
       </c>
       <c r="B114" s="11" t="s">
         <v>73</v>
@@ -8196,14 +8265,18 @@
         <v>85</v>
       </c>
       <c r="H114" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="I114" s="11"/>
-      <c r="J114" s="12"/>
+        <v>137</v>
+      </c>
+      <c r="I114" s="11">
+        <v>0.5</v>
+      </c>
+      <c r="J114" s="12" t="s">
+        <v>417</v>
+      </c>
     </row>
     <row r="115" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115" s="11" t="s">
-        <v>408</v>
+        <v>418</v>
       </c>
       <c r="B115" s="11" t="s">
         <v>73</v>
@@ -8231,7 +8304,7 @@
     </row>
     <row r="116" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="11" t="s">
-        <v>409</v>
+        <v>419</v>
       </c>
       <c r="B116" s="11" t="s">
         <v>73</v>
@@ -8259,7 +8332,7 @@
     </row>
     <row r="117" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="11" t="s">
-        <v>410</v>
+        <v>420</v>
       </c>
       <c r="B117" s="11" t="s">
         <v>78</v>
@@ -8268,7 +8341,7 @@
         <v>80</v>
       </c>
       <c r="D117" s="17" t="s">
-        <v>411</v>
+        <v>421</v>
       </c>
       <c r="E117" s="11" t="s">
         <v>199</v>
@@ -8286,12 +8359,12 @@
         <v>0.5</v>
       </c>
       <c r="J117" s="12" t="s">
-        <v>412</v>
+        <v>422</v>
       </c>
     </row>
     <row r="118" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A118" s="11" t="s">
-        <v>413</v>
+        <v>423</v>
       </c>
       <c r="B118" s="11" t="s">
         <v>78</v>
@@ -8300,7 +8373,7 @@
         <v>80</v>
       </c>
       <c r="D118" s="17" t="s">
-        <v>414</v>
+        <v>424</v>
       </c>
       <c r="E118" s="11" t="s">
         <v>199</v>
@@ -8318,12 +8391,12 @@
         <v>0.5</v>
       </c>
       <c r="J118" s="12" t="s">
-        <v>415</v>
+        <v>425</v>
       </c>
     </row>
     <row r="119" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119" s="11" t="s">
-        <v>416</v>
+        <v>426</v>
       </c>
       <c r="B119" s="11" t="s">
         <v>78</v>
@@ -8332,7 +8405,7 @@
         <v>80</v>
       </c>
       <c r="D119" s="17" t="s">
-        <v>417</v>
+        <v>427</v>
       </c>
       <c r="E119" s="11" t="s">
         <v>199</v>
@@ -8350,12 +8423,12 @@
         <v>0.5</v>
       </c>
       <c r="J119" s="12" t="s">
-        <v>418</v>
+        <v>428</v>
       </c>
     </row>
     <row r="120" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="11" t="s">
-        <v>419</v>
+        <v>429</v>
       </c>
       <c r="B120" s="11" t="s">
         <v>78</v>
@@ -8364,7 +8437,7 @@
         <v>80</v>
       </c>
       <c r="D120" s="17" t="s">
-        <v>420</v>
+        <v>430</v>
       </c>
       <c r="E120" s="11" t="s">
         <v>199</v>
@@ -8382,12 +8455,12 @@
         <v>0.5</v>
       </c>
       <c r="J120" s="12" t="s">
-        <v>421</v>
+        <v>431</v>
       </c>
     </row>
     <row r="121" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A121" s="11" t="s">
-        <v>422</v>
+        <v>432</v>
       </c>
       <c r="B121" s="11" t="s">
         <v>78</v>
@@ -8396,7 +8469,7 @@
         <v>80</v>
       </c>
       <c r="D121" s="17" t="s">
-        <v>423</v>
+        <v>433</v>
       </c>
       <c r="E121" s="11" t="s">
         <v>199</v>
@@ -8414,12 +8487,12 @@
         <v>0.5</v>
       </c>
       <c r="J121" s="12" t="s">
-        <v>424</v>
+        <v>434</v>
       </c>
     </row>
     <row r="122" spans="1:10" ht="55.15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="11" t="s">
-        <v>425</v>
+        <v>435</v>
       </c>
       <c r="B122" s="11" t="s">
         <v>78</v>
@@ -8428,7 +8501,7 @@
         <v>80</v>
       </c>
       <c r="D122" s="17" t="s">
-        <v>426</v>
+        <v>436</v>
       </c>
       <c r="E122" s="11" t="s">
         <v>263</v>
@@ -8446,12 +8519,12 @@
         <v>0.75</v>
       </c>
       <c r="J122" s="12" t="s">
-        <v>427</v>
+        <v>437</v>
       </c>
     </row>
     <row r="123" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A123" s="11" t="s">
-        <v>428</v>
+        <v>438</v>
       </c>
       <c r="B123" s="11" t="s">
         <v>78</v>
@@ -8460,7 +8533,7 @@
         <v>80</v>
       </c>
       <c r="D123" s="17" t="s">
-        <v>429</v>
+        <v>439</v>
       </c>
       <c r="E123" s="11" t="s">
         <v>263</v>
@@ -8478,12 +8551,12 @@
         <v>0.75</v>
       </c>
       <c r="J123" s="12" t="s">
-        <v>430</v>
+        <v>440</v>
       </c>
     </row>
     <row r="124" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A124" s="11" t="s">
-        <v>431</v>
+        <v>441</v>
       </c>
       <c r="B124" s="11" t="s">
         <v>78</v>
@@ -8492,7 +8565,7 @@
         <v>80</v>
       </c>
       <c r="D124" s="17" t="s">
-        <v>432</v>
+        <v>442</v>
       </c>
       <c r="E124" s="11" t="s">
         <v>24</v>
@@ -8510,12 +8583,12 @@
         <v>1.25</v>
       </c>
       <c r="J124" s="12" t="s">
-        <v>433</v>
+        <v>443</v>
       </c>
     </row>
     <row r="125" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125" s="11" t="s">
-        <v>434</v>
+        <v>444</v>
       </c>
       <c r="B125" s="11" t="s">
         <v>78</v>
@@ -8543,7 +8616,7 @@
     </row>
     <row r="126" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A126" s="11" t="s">
-        <v>435</v>
+        <v>445</v>
       </c>
       <c r="B126" s="11" t="s">
         <v>78</v>
@@ -8570,12 +8643,12 @@
         <v>0.5</v>
       </c>
       <c r="J126" s="12" t="s">
-        <v>436</v>
+        <v>446</v>
       </c>
     </row>
     <row r="127" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A127" s="11" t="s">
-        <v>437</v>
+        <v>447</v>
       </c>
       <c r="B127" s="11" t="s">
         <v>78</v>
@@ -8603,7 +8676,7 @@
     </row>
     <row r="128" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A128" s="11" t="s">
-        <v>438</v>
+        <v>448</v>
       </c>
       <c r="B128" s="11" t="s">
         <v>78</v>
@@ -8631,7 +8704,7 @@
     </row>
     <row r="129" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129" s="11" t="s">
-        <v>439</v>
+        <v>449</v>
       </c>
       <c r="B129" s="11" t="s">
         <v>87</v>
@@ -8640,7 +8713,7 @@
         <v>88</v>
       </c>
       <c r="D129" s="17" t="s">
-        <v>440</v>
+        <v>450</v>
       </c>
       <c r="E129" s="11" t="s">
         <v>199</v>
@@ -8659,7 +8732,7 @@
     </row>
     <row r="130" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" s="11" t="s">
-        <v>441</v>
+        <v>451</v>
       </c>
       <c r="B130" s="11" t="s">
         <v>87</v>
@@ -8668,7 +8741,7 @@
         <v>88</v>
       </c>
       <c r="D130" s="17" t="s">
-        <v>442</v>
+        <v>452</v>
       </c>
       <c r="E130" s="11" t="s">
         <v>199</v>
@@ -8687,7 +8760,7 @@
     </row>
     <row r="131" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="11" t="s">
-        <v>443</v>
+        <v>453</v>
       </c>
       <c r="B131" s="11" t="s">
         <v>87</v>
@@ -8696,7 +8769,7 @@
         <v>88</v>
       </c>
       <c r="D131" s="17" t="s">
-        <v>417</v>
+        <v>427</v>
       </c>
       <c r="E131" s="11" t="s">
         <v>199</v>
@@ -8715,7 +8788,7 @@
     </row>
     <row r="132" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132" s="11" t="s">
-        <v>444</v>
+        <v>454</v>
       </c>
       <c r="B132" s="11" t="s">
         <v>87</v>
@@ -8724,7 +8797,7 @@
         <v>88</v>
       </c>
       <c r="D132" s="17" t="s">
-        <v>445</v>
+        <v>455</v>
       </c>
       <c r="E132" s="11" t="s">
         <v>199</v>
@@ -8743,7 +8816,7 @@
     </row>
     <row r="133" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A133" s="11" t="s">
-        <v>446</v>
+        <v>456</v>
       </c>
       <c r="B133" s="11" t="s">
         <v>87</v>
@@ -8752,7 +8825,7 @@
         <v>88</v>
       </c>
       <c r="D133" s="17" t="s">
-        <v>447</v>
+        <v>457</v>
       </c>
       <c r="E133" s="11" t="s">
         <v>199</v>
@@ -8771,7 +8844,7 @@
     </row>
     <row r="134" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A134" s="11" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B134" s="11" t="s">
         <v>87</v>
@@ -8780,7 +8853,7 @@
         <v>88</v>
       </c>
       <c r="D134" s="17" t="s">
-        <v>449</v>
+        <v>459</v>
       </c>
       <c r="E134" s="11" t="s">
         <v>263</v>
@@ -8799,7 +8872,7 @@
     </row>
     <row r="135" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A135" s="11" t="s">
-        <v>450</v>
+        <v>460</v>
       </c>
       <c r="B135" s="11" t="s">
         <v>87</v>
@@ -8808,7 +8881,7 @@
         <v>88</v>
       </c>
       <c r="D135" s="17" t="s">
-        <v>429</v>
+        <v>439</v>
       </c>
       <c r="E135" s="11" t="s">
         <v>263</v>
@@ -8827,7 +8900,7 @@
     </row>
     <row r="136" spans="1:10" ht="55.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A136" s="11" t="s">
-        <v>451</v>
+        <v>461</v>
       </c>
       <c r="B136" s="11" t="s">
         <v>87</v>
@@ -8836,7 +8909,7 @@
         <v>88</v>
       </c>
       <c r="D136" s="17" t="s">
-        <v>452</v>
+        <v>462</v>
       </c>
       <c r="E136" s="11" t="s">
         <v>24</v>
@@ -8855,7 +8928,7 @@
     </row>
     <row r="137" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A137" s="11" t="s">
-        <v>453</v>
+        <v>463</v>
       </c>
       <c r="B137" s="11" t="s">
         <v>87</v>
@@ -8876,14 +8949,18 @@
         <v>85</v>
       </c>
       <c r="H137" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="I137" s="11"/>
-      <c r="J137" s="12"/>
+        <v>137</v>
+      </c>
+      <c r="I137" s="11">
+        <v>0.25</v>
+      </c>
+      <c r="J137" s="12" t="s">
+        <v>464</v>
+      </c>
     </row>
     <row r="138" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A138" s="11" t="s">
-        <v>454</v>
+        <v>465</v>
       </c>
       <c r="B138" s="11" t="s">
         <v>87</v>
@@ -8911,7 +8988,7 @@
     </row>
     <row r="139" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A139" s="11" t="s">
-        <v>455</v>
+        <v>466</v>
       </c>
       <c r="B139" s="11" t="s">
         <v>87</v>
@@ -8939,7 +9016,7 @@
     </row>
     <row r="140" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A140" s="11" t="s">
-        <v>456</v>
+        <v>467</v>
       </c>
       <c r="B140" s="11" t="s">
         <v>87</v>
@@ -8967,7 +9044,7 @@
     </row>
     <row r="141" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A141" s="11" t="s">
-        <v>457</v>
+        <v>468</v>
       </c>
       <c r="B141" s="11" t="s">
         <v>84</v>
@@ -8976,7 +9053,7 @@
         <v>93</v>
       </c>
       <c r="D141" s="17" t="s">
-        <v>411</v>
+        <v>421</v>
       </c>
       <c r="E141" s="11" t="s">
         <v>199</v>
@@ -8994,12 +9071,12 @@
         <v>0.75</v>
       </c>
       <c r="J141" s="12" t="s">
-        <v>458</v>
+        <v>469</v>
       </c>
     </row>
     <row r="142" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A142" s="11" t="s">
-        <v>459</v>
+        <v>470</v>
       </c>
       <c r="B142" s="11" t="s">
         <v>84</v>
@@ -9008,7 +9085,7 @@
         <v>93</v>
       </c>
       <c r="D142" s="17" t="s">
-        <v>460</v>
+        <v>471</v>
       </c>
       <c r="E142" s="11" t="s">
         <v>199</v>
@@ -9026,12 +9103,12 @@
         <v>0.5</v>
       </c>
       <c r="J142" s="12" t="s">
-        <v>461</v>
+        <v>472</v>
       </c>
     </row>
     <row r="143" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A143" s="11" t="s">
-        <v>462</v>
+        <v>473</v>
       </c>
       <c r="B143" s="11" t="s">
         <v>84</v>
@@ -9040,7 +9117,7 @@
         <v>93</v>
       </c>
       <c r="D143" s="17" t="s">
-        <v>463</v>
+        <v>474</v>
       </c>
       <c r="E143" s="11" t="s">
         <v>199</v>
@@ -9058,12 +9135,12 @@
         <v>0.5</v>
       </c>
       <c r="J143" s="12" t="s">
-        <v>464</v>
+        <v>475</v>
       </c>
     </row>
     <row r="144" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A144" s="11" t="s">
-        <v>465</v>
+        <v>476</v>
       </c>
       <c r="B144" s="11" t="s">
         <v>84</v>
@@ -9072,7 +9149,7 @@
         <v>93</v>
       </c>
       <c r="D144" s="17" t="s">
-        <v>466</v>
+        <v>477</v>
       </c>
       <c r="E144" s="11" t="s">
         <v>199</v>
@@ -9090,12 +9167,12 @@
         <v>0.5</v>
       </c>
       <c r="J144" s="12" t="s">
-        <v>467</v>
+        <v>478</v>
       </c>
     </row>
     <row r="145" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A145" s="11" t="s">
-        <v>468</v>
+        <v>479</v>
       </c>
       <c r="B145" s="11" t="s">
         <v>84</v>
@@ -9104,7 +9181,7 @@
         <v>93</v>
       </c>
       <c r="D145" s="17" t="s">
-        <v>423</v>
+        <v>433</v>
       </c>
       <c r="E145" s="11" t="s">
         <v>199</v>
@@ -9122,12 +9199,12 @@
         <v>0.5</v>
       </c>
       <c r="J145" s="12" t="s">
-        <v>469</v>
+        <v>480</v>
       </c>
     </row>
     <row r="146" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A146" s="11" t="s">
-        <v>470</v>
+        <v>481</v>
       </c>
       <c r="B146" s="11" t="s">
         <v>84</v>
@@ -9136,7 +9213,7 @@
         <v>93</v>
       </c>
       <c r="D146" s="17" t="s">
-        <v>471</v>
+        <v>482</v>
       </c>
       <c r="E146" s="11" t="s">
         <v>24</v>
@@ -9154,12 +9231,12 @@
         <v>0.75</v>
       </c>
       <c r="J146" s="12" t="s">
-        <v>472</v>
+        <v>483</v>
       </c>
     </row>
     <row r="147" spans="1:10" ht="151.9" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A147" s="11" t="s">
-        <v>473</v>
+        <v>484</v>
       </c>
       <c r="B147" s="11" t="s">
         <v>84</v>
@@ -9168,7 +9245,7 @@
         <v>93</v>
       </c>
       <c r="D147" s="17" t="s">
-        <v>474</v>
+        <v>485</v>
       </c>
       <c r="E147" s="11" t="s">
         <v>24</v>
@@ -9186,12 +9263,12 @@
         <v>0.75</v>
       </c>
       <c r="J147" s="12" t="s">
-        <v>475</v>
+        <v>486</v>
       </c>
     </row>
     <row r="148" spans="1:10" ht="55.15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A148" s="11" t="s">
-        <v>476</v>
+        <v>487</v>
       </c>
       <c r="B148" s="11" t="s">
         <v>84</v>
@@ -9218,12 +9295,12 @@
         <v>0.5</v>
       </c>
       <c r="J148" s="12" t="s">
-        <v>477</v>
+        <v>488</v>
       </c>
     </row>
     <row r="149" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A149" s="11" t="s">
-        <v>478</v>
+        <v>489</v>
       </c>
       <c r="B149" s="11" t="s">
         <v>84</v>
@@ -9251,7 +9328,7 @@
     </row>
     <row r="150" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A150" s="11" t="s">
-        <v>479</v>
+        <v>490</v>
       </c>
       <c r="B150" s="11" t="s">
         <v>84</v>
@@ -9279,7 +9356,7 @@
     </row>
     <row r="151" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A151" s="11" t="s">
-        <v>480</v>
+        <v>491</v>
       </c>
       <c r="B151" s="11" t="s">
         <v>98</v>
@@ -9288,7 +9365,7 @@
         <v>99</v>
       </c>
       <c r="D151" s="17" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="E151" s="11" t="s">
         <v>199</v>
@@ -9307,7 +9384,7 @@
     </row>
     <row r="152" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A152" s="11" t="s">
-        <v>481</v>
+        <v>492</v>
       </c>
       <c r="B152" s="11" t="s">
         <v>98</v>
@@ -9316,7 +9393,7 @@
         <v>99</v>
       </c>
       <c r="D152" s="17" t="s">
-        <v>482</v>
+        <v>493</v>
       </c>
       <c r="E152" s="11" t="s">
         <v>199</v>
@@ -9335,7 +9412,7 @@
     </row>
     <row r="153" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153" s="11" t="s">
-        <v>483</v>
+        <v>494</v>
       </c>
       <c r="B153" s="11" t="s">
         <v>98</v>
@@ -9344,7 +9421,7 @@
         <v>99</v>
       </c>
       <c r="D153" s="17" t="s">
-        <v>417</v>
+        <v>427</v>
       </c>
       <c r="E153" s="11" t="s">
         <v>199</v>
@@ -9362,12 +9439,12 @@
         <v>0.5</v>
       </c>
       <c r="J153" s="12" t="s">
-        <v>484</v>
+        <v>495</v>
       </c>
     </row>
     <row r="154" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A154" s="11" t="s">
-        <v>485</v>
+        <v>496</v>
       </c>
       <c r="B154" s="11" t="s">
         <v>98</v>
@@ -9376,7 +9453,7 @@
         <v>99</v>
       </c>
       <c r="D154" s="17" t="s">
-        <v>486</v>
+        <v>497</v>
       </c>
       <c r="E154" s="11" t="s">
         <v>199</v>
@@ -9395,7 +9472,7 @@
     </row>
     <row r="155" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A155" s="11" t="s">
-        <v>487</v>
+        <v>498</v>
       </c>
       <c r="B155" s="11" t="s">
         <v>98</v>
@@ -9404,7 +9481,7 @@
         <v>99</v>
       </c>
       <c r="D155" s="17" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="E155" s="11" t="s">
         <v>199</v>
@@ -9423,7 +9500,7 @@
     </row>
     <row r="156" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A156" s="11" t="s">
-        <v>488</v>
+        <v>499</v>
       </c>
       <c r="B156" s="11" t="s">
         <v>98</v>
@@ -9432,7 +9509,7 @@
         <v>99</v>
       </c>
       <c r="D156" s="17" t="s">
-        <v>489</v>
+        <v>500</v>
       </c>
       <c r="E156" s="11" t="s">
         <v>24</v>
@@ -9451,7 +9528,7 @@
     </row>
     <row r="157" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A157" s="11" t="s">
-        <v>490</v>
+        <v>501</v>
       </c>
       <c r="B157" s="11" t="s">
         <v>98</v>
@@ -9478,12 +9555,12 @@
         <v>0.25</v>
       </c>
       <c r="J157" s="12" t="s">
-        <v>491</v>
+        <v>502</v>
       </c>
     </row>
     <row r="158" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A158" s="11" t="s">
-        <v>492</v>
+        <v>503</v>
       </c>
       <c r="B158" s="11" t="s">
         <v>98</v>
@@ -9511,7 +9588,7 @@
     </row>
     <row r="159" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A159" s="11" t="s">
-        <v>493</v>
+        <v>504</v>
       </c>
       <c r="B159" s="11" t="s">
         <v>98</v>
@@ -9539,7 +9616,7 @@
     </row>
     <row r="160" spans="1:10" ht="55.15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A160" s="11" t="s">
-        <v>494</v>
+        <v>505</v>
       </c>
       <c r="B160" s="11" t="s">
         <v>102</v>
@@ -9548,7 +9625,7 @@
         <v>103</v>
       </c>
       <c r="D160" s="17" t="s">
-        <v>392</v>
+        <v>397</v>
       </c>
       <c r="E160" s="11" t="s">
         <v>199</v>
@@ -9566,12 +9643,12 @@
         <v>0.75</v>
       </c>
       <c r="J160" s="12" t="s">
-        <v>495</v>
+        <v>506</v>
       </c>
     </row>
     <row r="161" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A161" s="11" t="s">
-        <v>496</v>
+        <v>507</v>
       </c>
       <c r="B161" s="11" t="s">
         <v>102</v>
@@ -9580,7 +9657,7 @@
         <v>103</v>
       </c>
       <c r="D161" s="17" t="s">
-        <v>497</v>
+        <v>508</v>
       </c>
       <c r="E161" s="11" t="s">
         <v>199</v>
@@ -9599,7 +9676,7 @@
     </row>
     <row r="162" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A162" s="11" t="s">
-        <v>498</v>
+        <v>509</v>
       </c>
       <c r="B162" s="11" t="s">
         <v>102</v>
@@ -9608,7 +9685,7 @@
         <v>103</v>
       </c>
       <c r="D162" s="17" t="s">
-        <v>499</v>
+        <v>510</v>
       </c>
       <c r="E162" s="11" t="s">
         <v>199</v>
@@ -9627,7 +9704,7 @@
     </row>
     <row r="163" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A163" s="11" t="s">
-        <v>500</v>
+        <v>511</v>
       </c>
       <c r="B163" s="11" t="s">
         <v>102</v>
@@ -9636,7 +9713,7 @@
         <v>103</v>
       </c>
       <c r="D163" s="17" t="s">
-        <v>400</v>
+        <v>406</v>
       </c>
       <c r="E163" s="11" t="s">
         <v>199</v>
@@ -9654,12 +9731,12 @@
         <v>0.5</v>
       </c>
       <c r="J163" s="12" t="s">
-        <v>501</v>
+        <v>512</v>
       </c>
     </row>
     <row r="164" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A164" s="11" t="s">
-        <v>502</v>
+        <v>513</v>
       </c>
       <c r="B164" s="11" t="s">
         <v>102</v>
@@ -9668,7 +9745,7 @@
         <v>103</v>
       </c>
       <c r="D164" s="17" t="s">
-        <v>503</v>
+        <v>514</v>
       </c>
       <c r="E164" s="11" t="s">
         <v>24</v>
@@ -9686,12 +9763,12 @@
         <v>1.5</v>
       </c>
       <c r="J164" s="12" t="s">
-        <v>504</v>
+        <v>515</v>
       </c>
     </row>
     <row r="165" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A165" s="11" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="B165" s="11" t="s">
         <v>102</v>
@@ -9719,7 +9796,7 @@
     </row>
     <row r="166" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A166" s="11" t="s">
-        <v>506</v>
+        <v>517</v>
       </c>
       <c r="B166" s="11" t="s">
         <v>102</v>
@@ -9747,7 +9824,7 @@
     </row>
     <row r="167" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A167" s="11" t="s">
-        <v>507</v>
+        <v>518</v>
       </c>
       <c r="B167" s="11" t="s">
         <v>102</v>
@@ -9775,7 +9852,7 @@
     </row>
     <row r="168" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A168" s="11" t="s">
-        <v>508</v>
+        <v>519</v>
       </c>
       <c r="B168" s="11" t="s">
         <v>96</v>
@@ -9784,7 +9861,7 @@
         <v>107</v>
       </c>
       <c r="D168" s="17" t="s">
-        <v>509</v>
+        <v>520</v>
       </c>
       <c r="E168" s="11" t="s">
         <v>199</v>
@@ -9802,12 +9879,12 @@
         <v>0.5</v>
       </c>
       <c r="J168" s="12" t="s">
-        <v>510</v>
+        <v>521</v>
       </c>
     </row>
     <row r="169" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A169" s="11" t="s">
-        <v>511</v>
+        <v>522</v>
       </c>
       <c r="B169" s="11" t="s">
         <v>96</v>
@@ -9816,7 +9893,7 @@
         <v>107</v>
       </c>
       <c r="D169" s="17" t="s">
-        <v>512</v>
+        <v>523</v>
       </c>
       <c r="E169" s="11" t="s">
         <v>199</v>
@@ -9834,12 +9911,12 @@
         <v>0.5</v>
       </c>
       <c r="J169" s="12" t="s">
-        <v>513</v>
+        <v>524</v>
       </c>
     </row>
     <row r="170" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A170" s="11" t="s">
-        <v>514</v>
+        <v>525</v>
       </c>
       <c r="B170" s="11" t="s">
         <v>96</v>
@@ -9848,7 +9925,7 @@
         <v>107</v>
       </c>
       <c r="D170" s="17" t="s">
-        <v>515</v>
+        <v>526</v>
       </c>
       <c r="E170" s="11" t="s">
         <v>199</v>
@@ -9866,12 +9943,12 @@
         <v>0.5</v>
       </c>
       <c r="J170" s="12" t="s">
-        <v>516</v>
+        <v>527</v>
       </c>
     </row>
     <row r="171" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A171" s="11" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="B171" s="11" t="s">
         <v>96</v>
@@ -9880,7 +9957,7 @@
         <v>107</v>
       </c>
       <c r="D171" s="17" t="s">
-        <v>518</v>
+        <v>529</v>
       </c>
       <c r="E171" s="11" t="s">
         <v>199</v>
@@ -9898,12 +9975,12 @@
         <v>0.5</v>
       </c>
       <c r="J171" s="12" t="s">
-        <v>519</v>
+        <v>530</v>
       </c>
     </row>
     <row r="172" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A172" s="11" t="s">
-        <v>520</v>
+        <v>531</v>
       </c>
       <c r="B172" s="11" t="s">
         <v>96</v>
@@ -9912,7 +9989,7 @@
         <v>107</v>
       </c>
       <c r="D172" s="17" t="s">
-        <v>521</v>
+        <v>532</v>
       </c>
       <c r="E172" s="11" t="s">
         <v>199</v>
@@ -9930,12 +10007,12 @@
         <v>0.5</v>
       </c>
       <c r="J172" s="12" t="s">
-        <v>522</v>
+        <v>533</v>
       </c>
     </row>
     <row r="173" spans="1:10" ht="55.15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A173" s="11" t="s">
-        <v>523</v>
+        <v>534</v>
       </c>
       <c r="B173" s="11" t="s">
         <v>96</v>
@@ -9944,7 +10021,7 @@
         <v>107</v>
       </c>
       <c r="D173" s="17" t="s">
-        <v>524</v>
+        <v>535</v>
       </c>
       <c r="E173" s="11" t="s">
         <v>199</v>
@@ -9962,12 +10039,12 @@
         <v>0.25</v>
       </c>
       <c r="J173" s="12" t="s">
-        <v>525</v>
+        <v>536</v>
       </c>
     </row>
     <row r="174" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A174" s="11" t="s">
-        <v>526</v>
+        <v>537</v>
       </c>
       <c r="B174" s="11" t="s">
         <v>96</v>
@@ -9976,7 +10053,7 @@
         <v>107</v>
       </c>
       <c r="D174" s="17" t="s">
-        <v>527</v>
+        <v>538</v>
       </c>
       <c r="E174" s="11" t="s">
         <v>24</v>
@@ -9994,12 +10071,12 @@
         <v>0.5</v>
       </c>
       <c r="J174" s="12" t="s">
-        <v>528</v>
+        <v>539</v>
       </c>
     </row>
     <row r="175" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A175" s="11" t="s">
-        <v>529</v>
+        <v>540</v>
       </c>
       <c r="B175" s="11" t="s">
         <v>96</v>
@@ -10008,7 +10085,7 @@
         <v>107</v>
       </c>
       <c r="D175" s="17" t="s">
-        <v>530</v>
+        <v>541</v>
       </c>
       <c r="E175" s="11" t="s">
         <v>24</v>
@@ -10026,12 +10103,12 @@
         <v>0.5</v>
       </c>
       <c r="J175" s="12" t="s">
-        <v>531</v>
+        <v>542</v>
       </c>
     </row>
     <row r="176" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A176" s="11" t="s">
-        <v>532</v>
+        <v>543</v>
       </c>
       <c r="B176" s="11" t="s">
         <v>96</v>
@@ -10058,12 +10135,12 @@
         <v>0.5</v>
       </c>
       <c r="J176" s="12" t="s">
-        <v>533</v>
+        <v>544</v>
       </c>
     </row>
     <row r="177" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A177" s="11" t="s">
-        <v>534</v>
+        <v>545</v>
       </c>
       <c r="B177" s="11" t="s">
         <v>96</v>
@@ -10090,12 +10167,12 @@
         <v>0.5</v>
       </c>
       <c r="J177" s="12" t="s">
-        <v>535</v>
+        <v>546</v>
       </c>
     </row>
     <row r="178" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A178" s="11" t="s">
-        <v>536</v>
+        <v>547</v>
       </c>
       <c r="B178" s="11" t="s">
         <v>96</v>
@@ -10123,7 +10200,7 @@
     </row>
     <row r="179" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A179" s="11" t="s">
-        <v>537</v>
+        <v>548</v>
       </c>
       <c r="B179" s="11" t="s">
         <v>96</v>
@@ -10151,7 +10228,7 @@
     </row>
     <row r="180" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A180" s="11" t="s">
-        <v>538</v>
+        <v>549</v>
       </c>
       <c r="B180" s="11" t="s">
         <v>112</v>
@@ -10160,7 +10237,7 @@
         <v>113</v>
       </c>
       <c r="D180" s="17" t="s">
-        <v>539</v>
+        <v>550</v>
       </c>
       <c r="E180" s="11" t="s">
         <v>199</v>
@@ -10178,12 +10255,12 @@
         <v>0.75</v>
       </c>
       <c r="J180" s="12" t="s">
-        <v>540</v>
+        <v>551</v>
       </c>
     </row>
     <row r="181" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A181" s="11" t="s">
-        <v>541</v>
+        <v>552</v>
       </c>
       <c r="B181" s="11" t="s">
         <v>112</v>
@@ -10192,7 +10269,7 @@
         <v>113</v>
       </c>
       <c r="D181" s="17" t="s">
-        <v>542</v>
+        <v>553</v>
       </c>
       <c r="E181" s="11" t="s">
         <v>199</v>
@@ -10210,12 +10287,12 @@
         <v>0.5</v>
       </c>
       <c r="J181" s="12" t="s">
-        <v>543</v>
+        <v>554</v>
       </c>
     </row>
     <row r="182" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A182" s="11" t="s">
-        <v>544</v>
+        <v>555</v>
       </c>
       <c r="B182" s="11" t="s">
         <v>112</v>
@@ -10224,7 +10301,7 @@
         <v>113</v>
       </c>
       <c r="D182" s="17" t="s">
-        <v>545</v>
+        <v>556</v>
       </c>
       <c r="E182" s="11" t="s">
         <v>199</v>
@@ -10242,12 +10319,12 @@
         <v>0.5</v>
       </c>
       <c r="J182" s="12" t="s">
-        <v>546</v>
+        <v>557</v>
       </c>
     </row>
     <row r="183" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A183" s="11" t="s">
-        <v>547</v>
+        <v>558</v>
       </c>
       <c r="B183" s="11" t="s">
         <v>112</v>
@@ -10256,7 +10333,7 @@
         <v>113</v>
       </c>
       <c r="D183" s="17" t="s">
-        <v>548</v>
+        <v>559</v>
       </c>
       <c r="E183" s="11" t="s">
         <v>199</v>
@@ -10274,12 +10351,12 @@
         <v>0.5</v>
       </c>
       <c r="J183" s="12" t="s">
-        <v>549</v>
+        <v>560</v>
       </c>
     </row>
     <row r="184" spans="1:10" ht="55.15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A184" s="11" t="s">
-        <v>550</v>
+        <v>561</v>
       </c>
       <c r="B184" s="11" t="s">
         <v>112</v>
@@ -10288,7 +10365,7 @@
         <v>113</v>
       </c>
       <c r="D184" s="17" t="s">
-        <v>551</v>
+        <v>562</v>
       </c>
       <c r="E184" s="11" t="s">
         <v>199</v>
@@ -10300,16 +10377,18 @@
         <v>85</v>
       </c>
       <c r="H184" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="I184" s="11"/>
+        <v>137</v>
+      </c>
+      <c r="I184" s="11">
+        <v>0.5</v>
+      </c>
       <c r="J184" s="12" t="s">
-        <v>552</v>
+        <v>563</v>
       </c>
     </row>
     <row r="185" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A185" s="11" t="s">
-        <v>553</v>
+        <v>564</v>
       </c>
       <c r="B185" s="11" t="s">
         <v>112</v>
@@ -10318,7 +10397,7 @@
         <v>113</v>
       </c>
       <c r="D185" s="17" t="s">
-        <v>554</v>
+        <v>565</v>
       </c>
       <c r="E185" s="11" t="s">
         <v>24</v>
@@ -10336,12 +10415,12 @@
         <v>0.75</v>
       </c>
       <c r="J185" s="12" t="s">
-        <v>555</v>
+        <v>566</v>
       </c>
     </row>
     <row r="186" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A186" s="11" t="s">
-        <v>556</v>
+        <v>567</v>
       </c>
       <c r="B186" s="11" t="s">
         <v>112</v>
@@ -10350,7 +10429,7 @@
         <v>113</v>
       </c>
       <c r="D186" s="17" t="s">
-        <v>557</v>
+        <v>568</v>
       </c>
       <c r="E186" s="11" t="s">
         <v>24</v>
@@ -10368,12 +10447,12 @@
         <v>0.75</v>
       </c>
       <c r="J186" s="12" t="s">
-        <v>558</v>
+        <v>569</v>
       </c>
     </row>
     <row r="187" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A187" s="11" t="s">
-        <v>559</v>
+        <v>570</v>
       </c>
       <c r="B187" s="11" t="s">
         <v>112</v>
@@ -10400,12 +10479,12 @@
         <v>0.5</v>
       </c>
       <c r="J187" s="12" t="s">
-        <v>560</v>
+        <v>571</v>
       </c>
     </row>
     <row r="188" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A188" s="11" t="s">
-        <v>561</v>
+        <v>572</v>
       </c>
       <c r="B188" s="11" t="s">
         <v>112</v>
@@ -10433,7 +10512,7 @@
     </row>
     <row r="189" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A189" s="11" t="s">
-        <v>562</v>
+        <v>573</v>
       </c>
       <c r="B189" s="11" t="s">
         <v>112</v>
@@ -10461,7 +10540,7 @@
     </row>
     <row r="190" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A190" s="11" t="s">
-        <v>563</v>
+        <v>574</v>
       </c>
       <c r="B190" s="11" t="s">
         <v>118</v>
@@ -10470,7 +10549,7 @@
         <v>119</v>
       </c>
       <c r="D190" s="17" t="s">
-        <v>564</v>
+        <v>575</v>
       </c>
       <c r="E190" s="11" t="s">
         <v>199</v>
@@ -10489,7 +10568,7 @@
     </row>
     <row r="191" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A191" s="11" t="s">
-        <v>565</v>
+        <v>576</v>
       </c>
       <c r="B191" s="11" t="s">
         <v>118</v>
@@ -10498,7 +10577,7 @@
         <v>119</v>
       </c>
       <c r="D191" s="17" t="s">
-        <v>566</v>
+        <v>577</v>
       </c>
       <c r="E191" s="11" t="s">
         <v>199</v>
@@ -10517,7 +10596,7 @@
     </row>
     <row r="192" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A192" s="11" t="s">
-        <v>567</v>
+        <v>578</v>
       </c>
       <c r="B192" s="11" t="s">
         <v>118</v>
@@ -10526,7 +10605,7 @@
         <v>119</v>
       </c>
       <c r="D192" s="17" t="s">
-        <v>568</v>
+        <v>579</v>
       </c>
       <c r="E192" s="11" t="s">
         <v>199</v>
@@ -10545,7 +10624,7 @@
     </row>
     <row r="193" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A193" s="11" t="s">
-        <v>569</v>
+        <v>580</v>
       </c>
       <c r="B193" s="11" t="s">
         <v>118</v>
@@ -10554,7 +10633,7 @@
         <v>119</v>
       </c>
       <c r="D193" s="17" t="s">
-        <v>570</v>
+        <v>581</v>
       </c>
       <c r="E193" s="11" t="s">
         <v>199</v>
@@ -10573,7 +10652,7 @@
     </row>
     <row r="194" spans="1:10" ht="55.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A194" s="11" t="s">
-        <v>571</v>
+        <v>582</v>
       </c>
       <c r="B194" s="11" t="s">
         <v>118</v>
@@ -10582,7 +10661,7 @@
         <v>119</v>
       </c>
       <c r="D194" s="17" t="s">
-        <v>572</v>
+        <v>583</v>
       </c>
       <c r="E194" s="11" t="s">
         <v>199</v>
@@ -10601,7 +10680,7 @@
     </row>
     <row r="195" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A195" s="11" t="s">
-        <v>573</v>
+        <v>584</v>
       </c>
       <c r="B195" s="11" t="s">
         <v>118</v>
@@ -10610,7 +10689,7 @@
         <v>119</v>
       </c>
       <c r="D195" s="17" t="s">
-        <v>574</v>
+        <v>585</v>
       </c>
       <c r="E195" s="11" t="s">
         <v>199</v>
@@ -10629,7 +10708,7 @@
     </row>
     <row r="196" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A196" s="11" t="s">
-        <v>575</v>
+        <v>586</v>
       </c>
       <c r="B196" s="11" t="s">
         <v>118</v>
@@ -10638,7 +10717,7 @@
         <v>119</v>
       </c>
       <c r="D196" s="17" t="s">
-        <v>576</v>
+        <v>587</v>
       </c>
       <c r="E196" s="11" t="s">
         <v>24</v>
@@ -10657,7 +10736,7 @@
     </row>
     <row r="197" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A197" s="11" t="s">
-        <v>577</v>
+        <v>588</v>
       </c>
       <c r="B197" s="11" t="s">
         <v>118</v>
@@ -10666,7 +10745,7 @@
         <v>119</v>
       </c>
       <c r="D197" s="17" t="s">
-        <v>578</v>
+        <v>589</v>
       </c>
       <c r="E197" s="11" t="s">
         <v>24</v>
@@ -10685,7 +10764,7 @@
     </row>
     <row r="198" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A198" s="11" t="s">
-        <v>579</v>
+        <v>590</v>
       </c>
       <c r="B198" s="11" t="s">
         <v>118</v>
@@ -10713,7 +10792,7 @@
     </row>
     <row r="199" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A199" s="11" t="s">
-        <v>580</v>
+        <v>591</v>
       </c>
       <c r="B199" s="11" t="s">
         <v>118</v>
@@ -10741,7 +10820,7 @@
     </row>
     <row r="200" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A200" s="11" t="s">
-        <v>581</v>
+        <v>592</v>
       </c>
       <c r="B200" s="11" t="s">
         <v>118</v>
@@ -10769,7 +10848,7 @@
     </row>
     <row r="201" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A201" s="11" t="s">
-        <v>582</v>
+        <v>593</v>
       </c>
       <c r="B201" s="11" t="s">
         <v>118</v>
@@ -10797,7 +10876,7 @@
     </row>
     <row r="202" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A202" s="11" t="s">
-        <v>583</v>
+        <v>594</v>
       </c>
       <c r="B202" s="11" t="s">
         <v>77</v>
@@ -10806,7 +10885,7 @@
         <v>123</v>
       </c>
       <c r="D202" s="17" t="s">
-        <v>584</v>
+        <v>595</v>
       </c>
       <c r="E202" s="11" t="s">
         <v>199</v>
@@ -10824,12 +10903,12 @@
         <v>0.5</v>
       </c>
       <c r="J202" s="12" t="s">
-        <v>585</v>
+        <v>596</v>
       </c>
     </row>
     <row r="203" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A203" s="11" t="s">
-        <v>586</v>
+        <v>597</v>
       </c>
       <c r="B203" s="11" t="s">
         <v>77</v>
@@ -10838,7 +10917,7 @@
         <v>123</v>
       </c>
       <c r="D203" s="17" t="s">
-        <v>587</v>
+        <v>598</v>
       </c>
       <c r="E203" s="11" t="s">
         <v>199</v>
@@ -10856,12 +10935,12 @@
         <v>0.5</v>
       </c>
       <c r="J203" s="12" t="s">
-        <v>588</v>
+        <v>599</v>
       </c>
     </row>
     <row r="204" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A204" s="11" t="s">
-        <v>589</v>
+        <v>600</v>
       </c>
       <c r="B204" s="11" t="s">
         <v>77</v>
@@ -10870,7 +10949,7 @@
         <v>123</v>
       </c>
       <c r="D204" s="17" t="s">
-        <v>590</v>
+        <v>601</v>
       </c>
       <c r="E204" s="11" t="s">
         <v>199</v>
@@ -10888,12 +10967,12 @@
         <v>0.5</v>
       </c>
       <c r="J204" s="12" t="s">
-        <v>591</v>
+        <v>602</v>
       </c>
     </row>
     <row r="205" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A205" s="11" t="s">
-        <v>592</v>
+        <v>603</v>
       </c>
       <c r="B205" s="11" t="s">
         <v>77</v>
@@ -10902,7 +10981,7 @@
         <v>123</v>
       </c>
       <c r="D205" s="17" t="s">
-        <v>593</v>
+        <v>604</v>
       </c>
       <c r="E205" s="11" t="s">
         <v>199</v>
@@ -10920,12 +10999,12 @@
         <v>0.5</v>
       </c>
       <c r="J205" s="12" t="s">
-        <v>594</v>
+        <v>605</v>
       </c>
     </row>
     <row r="206" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A206" s="11" t="s">
-        <v>595</v>
+        <v>606</v>
       </c>
       <c r="B206" s="11" t="s">
         <v>77</v>
@@ -10934,7 +11013,7 @@
         <v>123</v>
       </c>
       <c r="D206" s="17" t="s">
-        <v>596</v>
+        <v>607</v>
       </c>
       <c r="E206" s="11" t="s">
         <v>199</v>
@@ -10952,12 +11031,12 @@
         <v>0.5</v>
       </c>
       <c r="J206" s="12" t="s">
-        <v>597</v>
+        <v>608</v>
       </c>
     </row>
     <row r="207" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A207" s="11" t="s">
-        <v>598</v>
+        <v>609</v>
       </c>
       <c r="B207" s="11" t="s">
         <v>77</v>
@@ -10966,7 +11045,7 @@
         <v>123</v>
       </c>
       <c r="D207" s="17" t="s">
-        <v>599</v>
+        <v>610</v>
       </c>
       <c r="E207" s="11" t="s">
         <v>199</v>
@@ -10984,12 +11063,12 @@
         <v>0.25</v>
       </c>
       <c r="J207" s="12" t="s">
-        <v>600</v>
+        <v>611</v>
       </c>
     </row>
     <row r="208" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A208" s="11" t="s">
-        <v>601</v>
+        <v>612</v>
       </c>
       <c r="B208" s="11" t="s">
         <v>77</v>
@@ -10998,7 +11077,7 @@
         <v>123</v>
       </c>
       <c r="D208" s="17" t="s">
-        <v>602</v>
+        <v>613</v>
       </c>
       <c r="E208" s="11" t="s">
         <v>24</v>
@@ -11016,12 +11095,12 @@
         <v>0.5</v>
       </c>
       <c r="J208" s="12" t="s">
-        <v>603</v>
+        <v>614</v>
       </c>
     </row>
     <row r="209" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A209" s="11" t="s">
-        <v>604</v>
+        <v>615</v>
       </c>
       <c r="B209" s="11" t="s">
         <v>77</v>
@@ -11030,7 +11109,7 @@
         <v>123</v>
       </c>
       <c r="D209" s="17" t="s">
-        <v>605</v>
+        <v>616</v>
       </c>
       <c r="E209" s="11" t="s">
         <v>24</v>
@@ -11048,12 +11127,12 @@
         <v>0.5</v>
       </c>
       <c r="J209" s="12" t="s">
-        <v>606</v>
+        <v>617</v>
       </c>
     </row>
     <row r="210" spans="1:10" ht="55.15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A210" s="11" t="s">
-        <v>607</v>
+        <v>618</v>
       </c>
       <c r="B210" s="11" t="s">
         <v>77</v>
@@ -11080,12 +11159,12 @@
         <v>0.5</v>
       </c>
       <c r="J210" s="12" t="s">
-        <v>608</v>
+        <v>619</v>
       </c>
     </row>
     <row r="211" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A211" s="11" t="s">
-        <v>609</v>
+        <v>620</v>
       </c>
       <c r="B211" s="11" t="s">
         <v>77</v>
@@ -11112,12 +11191,12 @@
         <v>0.5</v>
       </c>
       <c r="J211" s="12" t="s">
-        <v>610</v>
+        <v>621</v>
       </c>
     </row>
     <row r="212" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A212" s="11" t="s">
-        <v>611</v>
+        <v>622</v>
       </c>
       <c r="B212" s="11" t="s">
         <v>77</v>
@@ -11144,12 +11223,12 @@
         <v>0.5</v>
       </c>
       <c r="J212" s="12" t="s">
-        <v>612</v>
+        <v>623</v>
       </c>
     </row>
     <row r="213" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A213" s="11" t="s">
-        <v>613</v>
+        <v>624</v>
       </c>
       <c r="B213" s="11" t="s">
         <v>77</v>
@@ -11176,12 +11255,12 @@
         <v>0.25</v>
       </c>
       <c r="J213" s="12" t="s">
-        <v>614</v>
+        <v>625</v>
       </c>
     </row>
     <row r="214" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A214" s="11" t="s">
-        <v>615</v>
+        <v>626</v>
       </c>
       <c r="B214" s="11" t="s">
         <v>128</v>
@@ -11190,7 +11269,7 @@
         <v>129</v>
       </c>
       <c r="D214" s="17" t="s">
-        <v>411</v>
+        <v>421</v>
       </c>
       <c r="E214" s="11" t="s">
         <v>199</v>
@@ -11208,12 +11287,12 @@
         <v>0.5</v>
       </c>
       <c r="J214" s="12" t="s">
-        <v>616</v>
+        <v>627</v>
       </c>
     </row>
     <row r="215" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A215" s="11" t="s">
-        <v>617</v>
+        <v>628</v>
       </c>
       <c r="B215" s="11" t="s">
         <v>128</v>
@@ -11222,7 +11301,7 @@
         <v>129</v>
       </c>
       <c r="D215" s="17" t="s">
-        <v>618</v>
+        <v>629</v>
       </c>
       <c r="E215" s="11" t="s">
         <v>199</v>
@@ -11241,7 +11320,7 @@
     </row>
     <row r="216" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A216" s="11" t="s">
-        <v>619</v>
+        <v>630</v>
       </c>
       <c r="B216" s="11" t="s">
         <v>128</v>
@@ -11250,7 +11329,7 @@
         <v>129</v>
       </c>
       <c r="D216" s="17" t="s">
-        <v>620</v>
+        <v>631</v>
       </c>
       <c r="E216" s="11" t="s">
         <v>199</v>
@@ -11269,7 +11348,7 @@
     </row>
     <row r="217" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A217" s="11" t="s">
-        <v>621</v>
+        <v>632</v>
       </c>
       <c r="B217" s="11" t="s">
         <v>128</v>
@@ -11278,7 +11357,7 @@
         <v>129</v>
       </c>
       <c r="D217" s="17" t="s">
-        <v>423</v>
+        <v>433</v>
       </c>
       <c r="E217" s="11" t="s">
         <v>199</v>
@@ -11296,12 +11375,12 @@
         <v>0.25</v>
       </c>
       <c r="J217" s="12" t="s">
-        <v>622</v>
+        <v>633</v>
       </c>
     </row>
     <row r="218" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A218" s="11" t="s">
-        <v>623</v>
+        <v>634</v>
       </c>
       <c r="B218" s="11" t="s">
         <v>128</v>
@@ -11310,7 +11389,7 @@
         <v>129</v>
       </c>
       <c r="D218" s="17" t="s">
-        <v>624</v>
+        <v>635</v>
       </c>
       <c r="E218" s="11" t="s">
         <v>24</v>
@@ -11328,12 +11407,12 @@
         <v>0.75</v>
       </c>
       <c r="J218" s="12" t="s">
-        <v>625</v>
+        <v>636</v>
       </c>
     </row>
     <row r="219" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A219" s="11" t="s">
-        <v>626</v>
+        <v>637</v>
       </c>
       <c r="B219" s="11" t="s">
         <v>128</v>
@@ -11360,12 +11439,12 @@
         <v>0.25</v>
       </c>
       <c r="J219" s="12" t="s">
-        <v>627</v>
+        <v>638</v>
       </c>
     </row>
     <row r="220" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A220" s="11" t="s">
-        <v>628</v>
+        <v>639</v>
       </c>
       <c r="B220" s="11" t="s">
         <v>128</v>
@@ -11393,7 +11472,7 @@
     </row>
     <row r="221" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A221" s="11" t="s">
-        <v>629</v>
+        <v>640</v>
       </c>
       <c r="B221" s="11" t="s">
         <v>128</v>
@@ -11421,7 +11500,7 @@
     </row>
     <row r="222" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A222" s="11" t="s">
-        <v>630</v>
+        <v>641</v>
       </c>
       <c r="B222" s="11" t="s">
         <v>132</v>
@@ -11430,7 +11509,7 @@
         <v>133</v>
       </c>
       <c r="D222" s="17" t="s">
-        <v>631</v>
+        <v>642</v>
       </c>
       <c r="E222" s="11" t="s">
         <v>199</v>
@@ -11449,7 +11528,7 @@
     </row>
     <row r="223" spans="1:10" ht="55.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A223" s="11" t="s">
-        <v>632</v>
+        <v>643</v>
       </c>
       <c r="B223" s="11" t="s">
         <v>132</v>
@@ -11458,7 +11537,7 @@
         <v>133</v>
       </c>
       <c r="D223" s="17" t="s">
-        <v>633</v>
+        <v>644</v>
       </c>
       <c r="E223" s="11" t="s">
         <v>199</v>
@@ -11477,7 +11556,7 @@
     </row>
     <row r="224" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A224" s="11" t="s">
-        <v>634</v>
+        <v>645</v>
       </c>
       <c r="B224" s="11" t="s">
         <v>132</v>
@@ -11486,7 +11565,7 @@
         <v>133</v>
       </c>
       <c r="D224" s="17" t="s">
-        <v>635</v>
+        <v>646</v>
       </c>
       <c r="E224" s="11" t="s">
         <v>199</v>
@@ -11505,7 +11584,7 @@
     </row>
     <row r="225" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A225" s="11" t="s">
-        <v>636</v>
+        <v>647</v>
       </c>
       <c r="B225" s="11" t="s">
         <v>132</v>
@@ -11514,7 +11593,7 @@
         <v>133</v>
       </c>
       <c r="D225" s="17" t="s">
-        <v>637</v>
+        <v>648</v>
       </c>
       <c r="E225" s="11" t="s">
         <v>199</v>
@@ -11533,7 +11612,7 @@
     </row>
     <row r="226" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A226" s="11" t="s">
-        <v>638</v>
+        <v>649</v>
       </c>
       <c r="B226" s="11" t="s">
         <v>132</v>
@@ -11542,7 +11621,7 @@
         <v>133</v>
       </c>
       <c r="D226" s="17" t="s">
-        <v>639</v>
+        <v>650</v>
       </c>
       <c r="E226" s="11" t="s">
         <v>199</v>
@@ -11561,7 +11640,7 @@
     </row>
     <row r="227" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A227" s="11" t="s">
-        <v>640</v>
+        <v>651</v>
       </c>
       <c r="B227" s="11" t="s">
         <v>132</v>
@@ -11570,7 +11649,7 @@
         <v>133</v>
       </c>
       <c r="D227" s="17" t="s">
-        <v>641</v>
+        <v>652</v>
       </c>
       <c r="E227" s="11" t="s">
         <v>199</v>
@@ -11589,7 +11668,7 @@
     </row>
     <row r="228" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A228" s="11" t="s">
-        <v>642</v>
+        <v>653</v>
       </c>
       <c r="B228" s="11" t="s">
         <v>132</v>
@@ -11598,7 +11677,7 @@
         <v>133</v>
       </c>
       <c r="D228" s="17" t="s">
-        <v>643</v>
+        <v>654</v>
       </c>
       <c r="E228" s="11" t="s">
         <v>24</v>
@@ -11617,7 +11696,7 @@
     </row>
     <row r="229" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A229" s="11" t="s">
-        <v>644</v>
+        <v>655</v>
       </c>
       <c r="B229" s="11" t="s">
         <v>132</v>
@@ -11626,7 +11705,7 @@
         <v>133</v>
       </c>
       <c r="D229" s="17" t="s">
-        <v>645</v>
+        <v>656</v>
       </c>
       <c r="E229" s="11" t="s">
         <v>24</v>
@@ -11645,7 +11724,7 @@
     </row>
     <row r="230" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A230" s="11" t="s">
-        <v>646</v>
+        <v>657</v>
       </c>
       <c r="B230" s="11" t="s">
         <v>132</v>
@@ -11673,7 +11752,7 @@
     </row>
     <row r="231" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A231" s="11" t="s">
-        <v>647</v>
+        <v>658</v>
       </c>
       <c r="B231" s="11" t="s">
         <v>132</v>
@@ -11701,7 +11780,7 @@
     </row>
     <row r="232" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A232" s="11" t="s">
-        <v>648</v>
+        <v>659</v>
       </c>
       <c r="B232" s="11" t="s">
         <v>132</v>
@@ -11729,7 +11808,7 @@
     </row>
     <row r="233" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A233" s="11" t="s">
-        <v>649</v>
+        <v>660</v>
       </c>
       <c r="B233" s="11" t="s">
         <v>132</v>
@@ -11757,7 +11836,7 @@
     </row>
     <row r="234" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A234" s="11" t="s">
-        <v>650</v>
+        <v>661</v>
       </c>
       <c r="B234" s="11" t="s">
         <v>126</v>
@@ -11766,7 +11845,7 @@
         <v>139</v>
       </c>
       <c r="D234" s="17" t="s">
-        <v>651</v>
+        <v>662</v>
       </c>
       <c r="E234" s="11" t="s">
         <v>199</v>
@@ -11785,7 +11864,7 @@
     </row>
     <row r="235" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A235" s="11" t="s">
-        <v>652</v>
+        <v>663</v>
       </c>
       <c r="B235" s="11" t="s">
         <v>126</v>
@@ -11794,7 +11873,7 @@
         <v>139</v>
       </c>
       <c r="D235" s="17" t="s">
-        <v>653</v>
+        <v>664</v>
       </c>
       <c r="E235" s="11" t="s">
         <v>199</v>
@@ -11813,7 +11892,7 @@
     </row>
     <row r="236" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A236" s="11" t="s">
-        <v>654</v>
+        <v>665</v>
       </c>
       <c r="B236" s="11" t="s">
         <v>126</v>
@@ -11822,7 +11901,7 @@
         <v>139</v>
       </c>
       <c r="D236" s="17" t="s">
-        <v>655</v>
+        <v>666</v>
       </c>
       <c r="E236" s="11" t="s">
         <v>199</v>
@@ -11841,7 +11920,7 @@
     </row>
     <row r="237" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A237" s="11" t="s">
-        <v>656</v>
+        <v>667</v>
       </c>
       <c r="B237" s="11" t="s">
         <v>126</v>
@@ -11850,7 +11929,7 @@
         <v>139</v>
       </c>
       <c r="D237" s="17" t="s">
-        <v>657</v>
+        <v>668</v>
       </c>
       <c r="E237" s="11" t="s">
         <v>199</v>
@@ -11869,7 +11948,7 @@
     </row>
     <row r="238" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A238" s="11" t="s">
-        <v>658</v>
+        <v>669</v>
       </c>
       <c r="B238" s="11" t="s">
         <v>126</v>
@@ -11878,7 +11957,7 @@
         <v>139</v>
       </c>
       <c r="D238" s="17" t="s">
-        <v>659</v>
+        <v>670</v>
       </c>
       <c r="E238" s="11" t="s">
         <v>199</v>
@@ -11897,7 +11976,7 @@
     </row>
     <row r="239" spans="1:10" ht="55.15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A239" s="11" t="s">
-        <v>660</v>
+        <v>671</v>
       </c>
       <c r="B239" s="11" t="s">
         <v>126</v>
@@ -11906,7 +11985,7 @@
         <v>139</v>
       </c>
       <c r="D239" s="17" t="s">
-        <v>661</v>
+        <v>672</v>
       </c>
       <c r="E239" s="11" t="s">
         <v>199</v>
@@ -11925,7 +12004,7 @@
     </row>
     <row r="240" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A240" s="11" t="s">
-        <v>662</v>
+        <v>673</v>
       </c>
       <c r="B240" s="11" t="s">
         <v>126</v>
@@ -11934,7 +12013,7 @@
         <v>139</v>
       </c>
       <c r="D240" s="17" t="s">
-        <v>663</v>
+        <v>674</v>
       </c>
       <c r="E240" s="11" t="s">
         <v>24</v>
@@ -11953,7 +12032,7 @@
     </row>
     <row r="241" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A241" s="11" t="s">
-        <v>664</v>
+        <v>675</v>
       </c>
       <c r="B241" s="11" t="s">
         <v>126</v>
@@ -11962,7 +12041,7 @@
         <v>139</v>
       </c>
       <c r="D241" s="17" t="s">
-        <v>665</v>
+        <v>676</v>
       </c>
       <c r="E241" s="11" t="s">
         <v>24</v>
@@ -11981,7 +12060,7 @@
     </row>
     <row r="242" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A242" s="11" t="s">
-        <v>666</v>
+        <v>677</v>
       </c>
       <c r="B242" s="11" t="s">
         <v>126</v>
@@ -12009,7 +12088,7 @@
     </row>
     <row r="243" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A243" s="11" t="s">
-        <v>667</v>
+        <v>678</v>
       </c>
       <c r="B243" s="11" t="s">
         <v>126</v>
@@ -12037,7 +12116,7 @@
     </row>
     <row r="244" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A244" s="11" t="s">
-        <v>668</v>
+        <v>679</v>
       </c>
       <c r="B244" s="11" t="s">
         <v>126</v>
@@ -12065,7 +12144,7 @@
     </row>
     <row r="245" spans="1:10" ht="41.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A245" s="11" t="s">
-        <v>669</v>
+        <v>680</v>
       </c>
       <c r="B245" s="11" t="s">
         <v>126</v>
@@ -12093,7 +12172,7 @@
     </row>
     <row r="246" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A246" s="11" t="s">
-        <v>670</v>
+        <v>681</v>
       </c>
       <c r="B246" s="11" t="s">
         <v>143</v>
@@ -12102,7 +12181,7 @@
         <v>144</v>
       </c>
       <c r="D246" s="17" t="s">
-        <v>671</v>
+        <v>682</v>
       </c>
       <c r="E246" s="11" t="s">
         <v>199</v>
@@ -12121,7 +12200,7 @@
     </row>
     <row r="247" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A247" s="11" t="s">
-        <v>672</v>
+        <v>683</v>
       </c>
       <c r="B247" s="11" t="s">
         <v>143</v>
@@ -12130,7 +12209,7 @@
         <v>144</v>
       </c>
       <c r="D247" s="17" t="s">
-        <v>673</v>
+        <v>684</v>
       </c>
       <c r="E247" s="11" t="s">
         <v>199</v>
@@ -12149,7 +12228,7 @@
     </row>
     <row r="248" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A248" s="11" t="s">
-        <v>674</v>
+        <v>685</v>
       </c>
       <c r="B248" s="11" t="s">
         <v>143</v>
@@ -12158,7 +12237,7 @@
         <v>144</v>
       </c>
       <c r="D248" s="17" t="s">
-        <v>675</v>
+        <v>686</v>
       </c>
       <c r="E248" s="11" t="s">
         <v>199</v>
@@ -12177,7 +12256,7 @@
     </row>
     <row r="249" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A249" s="11" t="s">
-        <v>676</v>
+        <v>687</v>
       </c>
       <c r="B249" s="11" t="s">
         <v>143</v>
@@ -12186,7 +12265,7 @@
         <v>144</v>
       </c>
       <c r="D249" s="17" t="s">
-        <v>677</v>
+        <v>688</v>
       </c>
       <c r="E249" s="11" t="s">
         <v>199</v>
@@ -12205,7 +12284,7 @@
     </row>
     <row r="250" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A250" s="11" t="s">
-        <v>678</v>
+        <v>689</v>
       </c>
       <c r="B250" s="11" t="s">
         <v>143</v>
@@ -12214,7 +12293,7 @@
         <v>144</v>
       </c>
       <c r="D250" s="17" t="s">
-        <v>679</v>
+        <v>690</v>
       </c>
       <c r="E250" s="11" t="s">
         <v>199</v>
@@ -12233,7 +12312,7 @@
     </row>
     <row r="251" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A251" s="11" t="s">
-        <v>680</v>
+        <v>691</v>
       </c>
       <c r="B251" s="11" t="s">
         <v>143</v>
@@ -12242,7 +12321,7 @@
         <v>144</v>
       </c>
       <c r="D251" s="17" t="s">
-        <v>681</v>
+        <v>692</v>
       </c>
       <c r="E251" s="11" t="s">
         <v>199</v>
@@ -12261,7 +12340,7 @@
     </row>
     <row r="252" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A252" s="11" t="s">
-        <v>682</v>
+        <v>693</v>
       </c>
       <c r="B252" s="11" t="s">
         <v>143</v>
@@ -12270,7 +12349,7 @@
         <v>144</v>
       </c>
       <c r="D252" s="17" t="s">
-        <v>683</v>
+        <v>694</v>
       </c>
       <c r="E252" s="11" t="s">
         <v>24</v>
@@ -12289,7 +12368,7 @@
     </row>
     <row r="253" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A253" s="11" t="s">
-        <v>684</v>
+        <v>695</v>
       </c>
       <c r="B253" s="11" t="s">
         <v>143</v>
@@ -12298,7 +12377,7 @@
         <v>144</v>
       </c>
       <c r="D253" s="17" t="s">
-        <v>685</v>
+        <v>696</v>
       </c>
       <c r="E253" s="11" t="s">
         <v>24</v>
@@ -12317,7 +12396,7 @@
     </row>
     <row r="254" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A254" s="11" t="s">
-        <v>686</v>
+        <v>697</v>
       </c>
       <c r="B254" s="11" t="s">
         <v>143</v>
@@ -12345,7 +12424,7 @@
     </row>
     <row r="255" spans="1:10" ht="55.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A255" s="11" t="s">
-        <v>687</v>
+        <v>698</v>
       </c>
       <c r="B255" s="11" t="s">
         <v>143</v>
@@ -12373,7 +12452,7 @@
     </row>
     <row r="256" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A256" s="11" t="s">
-        <v>688</v>
+        <v>699</v>
       </c>
       <c r="B256" s="11" t="s">
         <v>143</v>
@@ -12401,7 +12480,7 @@
     </row>
     <row r="257" spans="1:10" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A257" s="11" t="s">
-        <v>689</v>
+        <v>700</v>
       </c>
       <c r="B257" s="11" t="s">
         <v>143</v>
@@ -12553,7 +12632,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="19" t="s">
-        <v>690</v>
+        <v>701</v>
       </c>
       <c r="B1" s="20"/>
       <c r="C1" s="20"/>
@@ -12563,7 +12642,7 @@
     </row>
     <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="21" t="s">
-        <v>691</v>
+        <v>702</v>
       </c>
       <c r="B2" s="20"/>
       <c r="C2" s="20"/>
@@ -12579,16 +12658,16 @@
         <v>192</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>692</v>
+        <v>703</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>693</v>
+        <v>704</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>694</v>
+        <v>705</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>695</v>
+        <v>706</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
@@ -12602,13 +12681,13 @@
         <v>1</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>696</v>
+        <v>707</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>697</v>
+        <v>708</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>698</v>
+        <v>709</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -12622,13 +12701,13 @@
         <v>2</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>699</v>
+        <v>710</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>700</v>
+        <v>711</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>698</v>
+        <v>709</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
@@ -12642,13 +12721,13 @@
         <v>3</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>701</v>
+        <v>712</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>702</v>
+        <v>713</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>698</v>
+        <v>709</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
@@ -12662,13 +12741,13 @@
         <v>4</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>703</v>
+        <v>714</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>704</v>
+        <v>715</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>698</v>
+        <v>709</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -12682,13 +12761,13 @@
         <v>1</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>705</v>
+        <v>716</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>706</v>
+        <v>717</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>698</v>
+        <v>709</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -12702,13 +12781,13 @@
         <v>2</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>707</v>
+        <v>718</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>708</v>
+        <v>719</v>
       </c>
       <c r="F11" s="13" t="s">
-        <v>698</v>
+        <v>709</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
@@ -12722,13 +12801,13 @@
         <v>3</v>
       </c>
       <c r="D12" s="12" t="s">
+        <v>720</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>721</v>
+      </c>
+      <c r="F12" s="11" t="s">
         <v>709</v>
-      </c>
-      <c r="E12" s="12" t="s">
-        <v>710</v>
-      </c>
-      <c r="F12" s="11" t="s">
-        <v>698</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
@@ -12742,13 +12821,13 @@
         <v>1</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>711</v>
+        <v>722</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>712</v>
+        <v>723</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>713</v>
+        <v>724</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
@@ -12762,13 +12841,13 @@
         <v>2</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>714</v>
+        <v>725</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>715</v>
+        <v>726</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>713</v>
+        <v>724</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
@@ -12782,13 +12861,13 @@
         <v>3</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>716</v>
+        <v>727</v>
       </c>
       <c r="E15" s="14" t="s">
-        <v>717</v>
+        <v>728</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>713</v>
+        <v>724</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -12802,13 +12881,13 @@
         <v>1</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>718</v>
+        <v>729</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>719</v>
+        <v>730</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>698</v>
+        <v>709</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
@@ -12822,13 +12901,13 @@
         <v>2</v>
       </c>
       <c r="D17" s="14" t="s">
-        <v>720</v>
+        <v>731</v>
       </c>
       <c r="E17" s="14" t="s">
-        <v>721</v>
+        <v>732</v>
       </c>
       <c r="F17" s="13" t="s">
-        <v>698</v>
+        <v>709</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -12842,13 +12921,13 @@
         <v>3</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>722</v>
+        <v>733</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>723</v>
+        <v>734</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>698</v>
+        <v>709</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
@@ -12862,13 +12941,13 @@
         <v>1</v>
       </c>
       <c r="D19" s="14" t="s">
+        <v>735</v>
+      </c>
+      <c r="E19" s="14" t="s">
+        <v>736</v>
+      </c>
+      <c r="F19" s="13" t="s">
         <v>724</v>
-      </c>
-      <c r="E19" s="14" t="s">
-        <v>725</v>
-      </c>
-      <c r="F19" s="13" t="s">
-        <v>698</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -12882,13 +12961,13 @@
         <v>2</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>726</v>
+        <v>737</v>
       </c>
       <c r="E20" s="12" t="s">
-        <v>727</v>
+        <v>738</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>698</v>
+        <v>724</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -12902,13 +12981,13 @@
         <v>3</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>728</v>
+        <v>739</v>
       </c>
       <c r="E21" s="14" t="s">
-        <v>729</v>
+        <v>740</v>
       </c>
       <c r="F21" s="13" t="s">
-        <v>698</v>
+        <v>724</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
@@ -12922,13 +13001,13 @@
         <v>1</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>730</v>
+        <v>741</v>
       </c>
       <c r="E22" s="12" t="s">
-        <v>731</v>
+        <v>742</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>713</v>
+        <v>724</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -12942,13 +13021,13 @@
         <v>2</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>732</v>
+        <v>743</v>
       </c>
       <c r="E23" s="14" t="s">
-        <v>733</v>
+        <v>744</v>
       </c>
       <c r="F23" s="13" t="s">
-        <v>713</v>
+        <v>724</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -12962,13 +13041,13 @@
         <v>3</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>734</v>
+        <v>745</v>
       </c>
       <c r="E24" s="12" t="s">
-        <v>735</v>
+        <v>746</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>713</v>
+        <v>724</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -12982,13 +13061,13 @@
         <v>4</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>736</v>
+        <v>747</v>
       </c>
       <c r="E25" s="14" t="s">
-        <v>737</v>
+        <v>748</v>
       </c>
       <c r="F25" s="13" t="s">
-        <v>713</v>
+        <v>724</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
@@ -13002,13 +13081,13 @@
         <v>1</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>738</v>
+        <v>749</v>
       </c>
       <c r="E26" s="12" t="s">
-        <v>739</v>
+        <v>750</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>713</v>
+        <v>724</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -13022,13 +13101,13 @@
         <v>2</v>
       </c>
       <c r="D27" s="14" t="s">
-        <v>740</v>
+        <v>751</v>
       </c>
       <c r="E27" s="14" t="s">
-        <v>741</v>
+        <v>752</v>
       </c>
       <c r="F27" s="13" t="s">
-        <v>713</v>
+        <v>724</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
@@ -13042,13 +13121,13 @@
         <v>1</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>742</v>
+        <v>753</v>
       </c>
       <c r="E28" s="12" t="s">
-        <v>743</v>
+        <v>754</v>
       </c>
       <c r="F28" s="11" t="s">
-        <v>698</v>
+        <v>709</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -13062,13 +13141,13 @@
         <v>2</v>
       </c>
       <c r="D29" s="14" t="s">
-        <v>744</v>
+        <v>755</v>
       </c>
       <c r="E29" s="14" t="s">
-        <v>745</v>
+        <v>756</v>
       </c>
       <c r="F29" s="13" t="s">
-        <v>698</v>
+        <v>709</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -13082,13 +13161,13 @@
         <v>3</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>746</v>
+        <v>757</v>
       </c>
       <c r="E30" s="12" t="s">
-        <v>747</v>
+        <v>758</v>
       </c>
       <c r="F30" s="11" t="s">
-        <v>698</v>
+        <v>709</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -13102,13 +13181,13 @@
         <v>1</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>748</v>
+        <v>759</v>
       </c>
       <c r="E31" s="14" t="s">
-        <v>749</v>
+        <v>760</v>
       </c>
       <c r="F31" s="13" t="s">
-        <v>698</v>
+        <v>724</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
@@ -13122,13 +13201,13 @@
         <v>2</v>
       </c>
       <c r="D32" s="12" t="s">
-        <v>750</v>
+        <v>761</v>
       </c>
       <c r="E32" s="12" t="s">
-        <v>751</v>
+        <v>762</v>
       </c>
       <c r="F32" s="11" t="s">
-        <v>698</v>
+        <v>724</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -13142,13 +13221,13 @@
         <v>1</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>752</v>
+        <v>763</v>
       </c>
       <c r="E33" s="14" t="s">
-        <v>753</v>
+        <v>764</v>
       </c>
       <c r="F33" s="13" t="s">
-        <v>713</v>
+        <v>724</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -13162,13 +13241,13 @@
         <v>2</v>
       </c>
       <c r="D34" s="12" t="s">
-        <v>754</v>
+        <v>765</v>
       </c>
       <c r="E34" s="12" t="s">
-        <v>755</v>
+        <v>766</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>713</v>
+        <v>724</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -13182,13 +13261,13 @@
         <v>3</v>
       </c>
       <c r="D35" s="14" t="s">
-        <v>756</v>
+        <v>767</v>
       </c>
       <c r="E35" s="14" t="s">
-        <v>757</v>
+        <v>768</v>
       </c>
       <c r="F35" s="13" t="s">
-        <v>713</v>
+        <v>724</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -13202,13 +13281,13 @@
         <v>4</v>
       </c>
       <c r="D36" s="12" t="s">
-        <v>758</v>
+        <v>769</v>
       </c>
       <c r="E36" s="12" t="s">
-        <v>759</v>
+        <v>770</v>
       </c>
       <c r="F36" s="11" t="s">
-        <v>698</v>
+        <v>709</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
@@ -13222,13 +13301,13 @@
         <v>1</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>760</v>
+        <v>771</v>
       </c>
       <c r="E37" s="14" t="s">
-        <v>761</v>
+        <v>772</v>
       </c>
       <c r="F37" s="13" t="s">
-        <v>698</v>
+        <v>724</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
@@ -13242,13 +13321,13 @@
         <v>2</v>
       </c>
       <c r="D38" s="12" t="s">
-        <v>762</v>
+        <v>773</v>
       </c>
       <c r="E38" s="12" t="s">
-        <v>763</v>
+        <v>774</v>
       </c>
       <c r="F38" s="11" t="s">
-        <v>698</v>
+        <v>724</v>
       </c>
     </row>
     <row r="39" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
@@ -13262,13 +13341,13 @@
         <v>1</v>
       </c>
       <c r="D39" s="14" t="s">
-        <v>764</v>
+        <v>775</v>
       </c>
       <c r="E39" s="14" t="s">
-        <v>765</v>
+        <v>776</v>
       </c>
       <c r="F39" s="13" t="s">
-        <v>713</v>
+        <v>724</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
@@ -13282,13 +13361,13 @@
         <v>2</v>
       </c>
       <c r="D40" s="12" t="s">
-        <v>766</v>
+        <v>777</v>
       </c>
       <c r="E40" s="12" t="s">
-        <v>767</v>
+        <v>778</v>
       </c>
       <c r="F40" s="11" t="s">
-        <v>713</v>
+        <v>724</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
@@ -13302,13 +13381,13 @@
         <v>1</v>
       </c>
       <c r="D41" s="14" t="s">
-        <v>768</v>
+        <v>779</v>
       </c>
       <c r="E41" s="14" t="s">
-        <v>769</v>
+        <v>780</v>
       </c>
       <c r="F41" s="13" t="s">
-        <v>713</v>
+        <v>724</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -13322,13 +13401,13 @@
         <v>2</v>
       </c>
       <c r="D42" s="12" t="s">
-        <v>770</v>
+        <v>781</v>
       </c>
       <c r="E42" s="12" t="s">
-        <v>771</v>
+        <v>782</v>
       </c>
       <c r="F42" s="11" t="s">
-        <v>713</v>
+        <v>724</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
@@ -13342,13 +13421,13 @@
         <v>1</v>
       </c>
       <c r="D43" s="14" t="s">
-        <v>772</v>
+        <v>783</v>
       </c>
       <c r="E43" s="14" t="s">
-        <v>773</v>
+        <v>784</v>
       </c>
       <c r="F43" s="13" t="s">
-        <v>713</v>
+        <v>724</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -13362,13 +13441,13 @@
         <v>2</v>
       </c>
       <c r="D44" s="12" t="s">
-        <v>774</v>
+        <v>785</v>
       </c>
       <c r="E44" s="12" t="s">
-        <v>775</v>
+        <v>786</v>
       </c>
       <c r="F44" s="11" t="s">
-        <v>713</v>
+        <v>724</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -13382,13 +13461,13 @@
         <v>1</v>
       </c>
       <c r="D45" s="14" t="s">
-        <v>776</v>
+        <v>787</v>
       </c>
       <c r="E45" s="14" t="s">
-        <v>777</v>
+        <v>788</v>
       </c>
       <c r="F45" s="13" t="s">
-        <v>713</v>
+        <v>724</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
@@ -13402,13 +13481,13 @@
         <v>2</v>
       </c>
       <c r="D46" s="12" t="s">
-        <v>778</v>
+        <v>789</v>
       </c>
       <c r="E46" s="12" t="s">
-        <v>779</v>
+        <v>790</v>
       </c>
       <c r="F46" s="11" t="s">
-        <v>713</v>
+        <v>724</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -13422,13 +13501,13 @@
         <v>3</v>
       </c>
       <c r="D47" s="14" t="s">
-        <v>780</v>
+        <v>791</v>
       </c>
       <c r="E47" s="14" t="s">
-        <v>781</v>
+        <v>792</v>
       </c>
       <c r="F47" s="13" t="s">
-        <v>713</v>
+        <v>724</v>
       </c>
     </row>
     <row r="48" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
@@ -13442,13 +13521,13 @@
         <v>1</v>
       </c>
       <c r="D48" s="12" t="s">
-        <v>782</v>
+        <v>793</v>
       </c>
       <c r="E48" s="12" t="s">
-        <v>783</v>
+        <v>794</v>
       </c>
       <c r="F48" s="11" t="s">
-        <v>713</v>
+        <v>724</v>
       </c>
     </row>
     <row r="49" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
@@ -13462,13 +13541,13 @@
         <v>2</v>
       </c>
       <c r="D49" s="14" t="s">
-        <v>784</v>
+        <v>795</v>
       </c>
       <c r="E49" s="14" t="s">
-        <v>785</v>
+        <v>796</v>
       </c>
       <c r="F49" s="13" t="s">
-        <v>713</v>
+        <v>724</v>
       </c>
     </row>
     <row r="50" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
@@ -13482,13 +13561,13 @@
         <v>3</v>
       </c>
       <c r="D50" s="12" t="s">
-        <v>786</v>
+        <v>797</v>
       </c>
       <c r="E50" s="12" t="s">
-        <v>787</v>
+        <v>798</v>
       </c>
       <c r="F50" s="11" t="s">
-        <v>713</v>
+        <v>724</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -13502,13 +13581,13 @@
         <v>1</v>
       </c>
       <c r="D51" s="14" t="s">
-        <v>788</v>
+        <v>799</v>
       </c>
       <c r="E51" s="14" t="s">
-        <v>789</v>
+        <v>800</v>
       </c>
       <c r="F51" s="13" t="s">
-        <v>698</v>
+        <v>709</v>
       </c>
     </row>
     <row r="52" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
@@ -13522,13 +13601,13 @@
         <v>2</v>
       </c>
       <c r="D52" s="12" t="s">
-        <v>790</v>
+        <v>801</v>
       </c>
       <c r="E52" s="12" t="s">
-        <v>791</v>
+        <v>802</v>
       </c>
       <c r="F52" s="11" t="s">
-        <v>698</v>
+        <v>709</v>
       </c>
     </row>
     <row r="53" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -13542,13 +13621,13 @@
         <v>1</v>
       </c>
       <c r="D53" s="14" t="s">
-        <v>792</v>
+        <v>803</v>
       </c>
       <c r="E53" s="14" t="s">
-        <v>793</v>
+        <v>804</v>
       </c>
       <c r="F53" s="13" t="s">
-        <v>713</v>
+        <v>724</v>
       </c>
     </row>
     <row r="54" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -13562,13 +13641,13 @@
         <v>2</v>
       </c>
       <c r="D54" s="12" t="s">
-        <v>794</v>
+        <v>805</v>
       </c>
       <c r="E54" s="12" t="s">
-        <v>795</v>
+        <v>806</v>
       </c>
       <c r="F54" s="11" t="s">
-        <v>713</v>
+        <v>724</v>
       </c>
     </row>
     <row r="55" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -13582,13 +13661,13 @@
         <v>1</v>
       </c>
       <c r="D55" s="14" t="s">
-        <v>796</v>
+        <v>807</v>
       </c>
       <c r="E55" s="14" t="s">
-        <v>797</v>
+        <v>808</v>
       </c>
       <c r="F55" s="13" t="s">
-        <v>713</v>
+        <v>724</v>
       </c>
     </row>
     <row r="56" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
@@ -13602,13 +13681,13 @@
         <v>2</v>
       </c>
       <c r="D56" s="12" t="s">
-        <v>798</v>
+        <v>809</v>
       </c>
       <c r="E56" s="12" t="s">
-        <v>799</v>
+        <v>810</v>
       </c>
       <c r="F56" s="11" t="s">
-        <v>713</v>
+        <v>724</v>
       </c>
     </row>
     <row r="57" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
@@ -13622,13 +13701,13 @@
         <v>1</v>
       </c>
       <c r="D57" s="14" t="s">
-        <v>800</v>
+        <v>811</v>
       </c>
       <c r="E57" s="14" t="s">
-        <v>801</v>
+        <v>812</v>
       </c>
       <c r="F57" s="13" t="s">
-        <v>698</v>
+        <v>709</v>
       </c>
     </row>
     <row r="58" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -13642,13 +13721,13 @@
         <v>1</v>
       </c>
       <c r="D58" s="12" t="s">
-        <v>802</v>
+        <v>813</v>
       </c>
       <c r="E58" s="12" t="s">
-        <v>803</v>
+        <v>814</v>
       </c>
       <c r="F58" s="11" t="s">
-        <v>698</v>
+        <v>709</v>
       </c>
     </row>
     <row r="59" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -13662,13 +13741,13 @@
         <v>2</v>
       </c>
       <c r="D59" s="14" t="s">
-        <v>804</v>
+        <v>815</v>
       </c>
       <c r="E59" s="14" t="s">
-        <v>805</v>
+        <v>816</v>
       </c>
       <c r="F59" s="13" t="s">
-        <v>698</v>
+        <v>709</v>
       </c>
     </row>
     <row r="60" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
@@ -13682,13 +13761,13 @@
         <v>1</v>
       </c>
       <c r="D60" s="12" t="s">
-        <v>806</v>
+        <v>817</v>
       </c>
       <c r="E60" s="12" t="s">
-        <v>807</v>
+        <v>818</v>
       </c>
       <c r="F60" s="11" t="s">
-        <v>698</v>
+        <v>709</v>
       </c>
     </row>
     <row r="61" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -13702,13 +13781,13 @@
         <v>2</v>
       </c>
       <c r="D61" s="14" t="s">
-        <v>808</v>
+        <v>819</v>
       </c>
       <c r="E61" s="14" t="s">
-        <v>809</v>
+        <v>820</v>
       </c>
       <c r="F61" s="13" t="s">
-        <v>698</v>
+        <v>709</v>
       </c>
     </row>
   </sheetData>
@@ -13752,7 +13831,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="19" t="s">
-        <v>810</v>
+        <v>821</v>
       </c>
       <c r="B1" s="20"/>
       <c r="C1" s="20"/>
@@ -13760,7 +13839,7 @@
     </row>
     <row r="2" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="21" t="s">
-        <v>811</v>
+        <v>822</v>
       </c>
       <c r="B2" s="20"/>
       <c r="C2" s="20"/>
@@ -13768,16 +13847,16 @@
     </row>
     <row r="4" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
-        <v>692</v>
+        <v>703</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>812</v>
+        <v>823</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>813</v>
+        <v>824</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>814</v>
+        <v>825</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -13785,13 +13864,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>815</v>
+        <v>826</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>816</v>
+        <v>827</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>698</v>
+        <v>709</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -13802,10 +13881,10 @@
         <v>218</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>817</v>
+        <v>828</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>698</v>
+        <v>709</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -13813,13 +13892,13 @@
         <v>3</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>818</v>
+        <v>829</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>819</v>
+        <v>830</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>698</v>
+        <v>709</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -13827,13 +13906,13 @@
         <v>4</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>820</v>
+        <v>831</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>821</v>
+        <v>832</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>698</v>
+        <v>709</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -13841,13 +13920,13 @@
         <v>5</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>822</v>
+        <v>833</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>823</v>
+        <v>834</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>698</v>
+        <v>709</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -13855,13 +13934,13 @@
         <v>6</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>824</v>
+        <v>835</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>825</v>
+        <v>836</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>698</v>
+        <v>709</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -13869,13 +13948,13 @@
         <v>7</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>826</v>
+        <v>837</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>827</v>
+        <v>838</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>698</v>
+        <v>709</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -13886,10 +13965,10 @@
         <v>221</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>828</v>
+        <v>839</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>698</v>
+        <v>709</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -13897,13 +13976,13 @@
         <v>9</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>829</v>
+        <v>840</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>830</v>
+        <v>841</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>698</v>
+        <v>709</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -13914,15 +13993,15 @@
         <v>224</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>831</v>
+        <v>842</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>698</v>
+        <v>709</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="23" t="s">
-        <v>832</v>
+        <v>843</v>
       </c>
       <c r="B16" s="20"/>
       <c r="C16" s="20"/>

</xml_diff>

<commit_message>
Pruebas del Sprint 2 completo: historias de Emilio con evidencia y cuatro correcciones
- Informe de Pruebas S2 cubre todo el sprint (52 casos, 49 ok); los casos de
  las historias App pasan al manifiesto de S6.
- BD/239: SEL_ACTIVO filtra por tipo y subtipos (HU-030 #1).
- BD/240: UPD_ACTIVO rechaza que un activo cuelgue de su propio subactivo
  (HU-035 #4).
- Activos.aspx: filtro por tipo de activo; ActivoFicha: pestaña Componentes
  con el arbol; Posicion.aspx: confirmacion al ocupar una posicion ocupada.
- Backlog S2: criterios marcados, tareas de pruebas terminadas, historias
  HU-033/034/045/192 en revision.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S2.xlsx
+++ b/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S2.xlsx
@@ -1302,7 +1302,7 @@
       </c>
       <c r="P6" s="17" t="inlineStr">
         <is>
-          <t>Construida por Emilio Fuentes: alta del activo con su ficha técnica y código automático. Pantalla en Activos → Activos. PENDIENTE: prueba en navegador. || ACTUALIZACION 06-09-2026 (Emilio Fuentes): en editar activo se agrego la seccion DATOS TECNICOS, donde el usuario define los datos propios del activo con nombre + unidad + valor (boton '+ Agregar dato'); lo que se agrega aqui tambien queda como campo del tipo en Atributos tecnicos (sincronizacion en ambos sentidos), y cada dato guardado tiene una X para quitarlo. Se agrego adjuntar DOCUMENTOS (PDF/imagenes) ademas de la foto. En el listado se agrego filtro en cascada Planta -&gt; Area -&gt; Linea. Se registro la planta de Hamburgo (Hamburgo S.A. -&gt; Panaderia -&gt; Lineas 1 a 4) con 19 equipos: Modeladoras (Fritsch), Hornos (Alitech), Revolvedoras/Amasadoras (Escher) y Camaras BT/MT (Anaconda).</t>
+          <t>Pruebas S2 (17-09): criterios OK tras dos correcciones de Bryan: SEL_ACTIVO filtra por tipo y subtipos (bloque 239) y UPD_ACTIVO rechaza ciclos en la jerarquia (bloque 240). Construida por Emilio Fuentes: alta del activo con su ficha técnica y código automático. Pantalla en Activos → Activos. PENDIENTE: prueba en navegador. || ACTUALIZACION 06-09-2026 (Emilio Fuentes): en editar activo se agrego la seccion DATOS TECNICOS, donde el usuario define los datos propios del activo con nombre + unidad + valor (boton '+ Agregar dato'); lo que se agrega aqui tambien queda como campo del tipo en Atributos tecnicos (sincronizacion en ambos sentidos), y cada dato guardado tiene una X para quitarlo. Se agrego adjuntar DOCUMENTOS (PDF/imagenes) ademas de la foto. En el listado se agrego filtro en cascada Planta -&gt; Area -&gt; Linea. Se registro la planta de Hamburgo (Hamburgo S.A. -&gt; Panaderia -&gt; Lineas 1 a 4) con 19 equipos: Modeladoras (Fritsch), Hornos (Alitech), Revolvedoras/Amasadoras (Escher) y Camaras BT/MT (Anaconda).</t>
         </is>
       </c>
     </row>
@@ -1523,7 +1523,7 @@
       </c>
       <c r="P9" s="18" t="inlineStr">
         <is>
-          <t>Parte WEB terminada por Emilio Fuentes: ficha consolidada e historial del activo en Activos → Ficha e historial. PENDIENTE: el consumo desde la App (T móvil, no es mi alcance) y la prueba en navegador. || ACTUALIZACION 06-09-2026 (Emilio Fuentes): Ficha e historial usa la misma barra de busqueda estandar de Activos (Busqueda avanzada + Buscar + Planta/Area/Linea/Habilitado) sobre una lista de resultados. La pestania Atributos muestra los VALORES tecnicos capturados por ese activo (con su unidad), y la pestania Repuestos los repuestos del activo.</t>
+          <t>Pruebas S2 (17-09): #1 y #2 OK; #3 es de la app (Sprint 6). Parte WEB terminada por Emilio Fuentes: ficha consolidada e historial del activo en Activos → Ficha e historial. PENDIENTE: el consumo desde la App (T móvil, no es mi alcance) y la prueba en navegador. || ACTUALIZACION 06-09-2026 (Emilio Fuentes): Ficha e historial usa la misma barra de busqueda estandar de Activos (Busqueda avanzada + Buscar + Planta/Area/Linea/Habilitado) sobre una lista de resultados. La pestania Atributos muestra los VALORES tecnicos capturados por ese activo (con su unidad), y la pestania Repuestos los repuestos del activo.</t>
         </is>
       </c>
     </row>
@@ -1730,11 +1730,19 @@
       </c>
       <c r="N12" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="O12" s="12" t="n"/>
-      <c r="P12" s="12" t="n"/>
+          <t>En revisión</t>
+        </is>
+      </c>
+      <c r="O12" s="12" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
+      <c r="P12" s="12" t="inlineStr">
+        <is>
+          <t>Construida por Bryan Chávez (bloques 231-233). Evidencia S2 con los criterios OK. FALTA la verificacion de los criterios, que es de Catalina.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="69" customHeight="1" s="20">
       <c r="A13" s="13" t="inlineStr">
@@ -1807,7 +1815,7 @@
       </c>
       <c r="P13" s="18" t="inlineStr">
         <is>
-          <t>Construida por Emilio Fuentes: componentes del activo en Activos → Componentes, con jerarquía padre/hijo y código automático (COM). La baja rechaza si tiene subcomponentes. PENDIENTE: prueba en navegador. || ACTUALIZACION 06-09-2026 (Emilio Fuentes): se replanteo el alcance. Un componente de un activo es en la practica un REPUESTO y esos ya se administran en el modulo Repuestos, por lo que en la Ficha del activo la pestania 'Componentes' se reemplazo por 'Repuestos': ahora muestra los repuestos asignados/compatibles con ese activo. No se registran componentes en una pantalla aparte.</t>
+          <t>Pruebas S2 (17-09): #1 y #2 OK (la ficha del activo gano la pestaña Componentes con el arbol). #3 parcial: el estado cambia con fecha y usuario, pero sin motivo ni historial de estados del componente (base pendiente). Construida por Emilio Fuentes: componentes del activo en Activos → Componentes, con jerarquía padre/hijo y código automático (COM). La baja rechaza si tiene subcomponentes. PENDIENTE: prueba en navegador. || ACTUALIZACION 06-09-2026 (Emilio Fuentes): se replanteo el alcance. Un componente de un activo es en la practica un REPUESTO y esos ya se administran en el modulo Repuestos, por lo que en la Ficha del activo la pestania 'Componentes' se reemplazo por 'Repuestos': ahora muestra los repuestos asignados/compatibles con ese activo. No se registran componentes en una pantalla aparte.</t>
         </is>
       </c>
     </row>
@@ -2168,11 +2176,19 @@
       </c>
       <c r="N18" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="O18" s="12" t="n"/>
-      <c r="P18" s="12" t="n"/>
+          <t>En revisión</t>
+        </is>
+      </c>
+      <c r="O18" s="12" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
+      <c r="P18" s="12" t="inlineStr">
+        <is>
+          <t>Construida por Bryan Chávez (bloques 231-233). Evidencia S2 con los criterios OK. FALTA la verificacion de los criterios, que es de Catalina.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="69" customHeight="1" s="20">
       <c r="A19" s="13" t="inlineStr">
@@ -2235,11 +2251,19 @@
       </c>
       <c r="N19" s="13" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="O19" s="14" t="n"/>
-      <c r="P19" s="14" t="n"/>
+          <t>En revisión</t>
+        </is>
+      </c>
+      <c r="O19" s="14" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
+      <c r="P19" s="14" t="inlineStr">
+        <is>
+          <t>Construida por Bryan Chávez (bloques 231-233). Evidencia S2 con los criterios OK. FALTA la verificacion de los criterios, que es de Catalina.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="55.15" customHeight="1" s="20">
       <c r="A20" s="11" t="inlineStr">
@@ -2462,7 +2486,7 @@
       </c>
       <c r="P22" s="17" t="inlineStr">
         <is>
-          <t>Construida por Emilio Fuentes: árbol de tipos de activo con jerarquía en Activos → Tipos de activo, con código automático (TIP). PENDIENTE: prueba en navegador. || ACTUALIZACION 06-09-2026 (Emilio Fuentes): el listado de Tipos de activo es un arbol plegable (chevron por columna). Arranca colapsado (solo raices) y despliega por nivel sin parpadeo; se desactivo el ORDENAMIENTO por columna porque rompe la jerarquia (el paginado se mantiene, 25 por pagina).</t>
+          <t>Pruebas S2 (17-09): criterios OK tras dos correcciones de Bryan: SEL_ACTIVO filtra por tipo y subtipos (bloque 239) y UPD_ACTIVO rechaza ciclos en la jerarquia (bloque 240). Construida por Emilio Fuentes: árbol de tipos de activo con jerarquía en Activos → Tipos de activo, con código automático (TIP). PENDIENTE: prueba en navegador. || ACTUALIZACION 06-09-2026 (Emilio Fuentes): el listado de Tipos de activo es un arbol plegable (chevron por columna). Arranca colapsado (solo raices) y despliega por nivel sin parpadeo; se desactivo el ORDENAMIENTO por columna porque rompe la jerarquia (el paginado se mantiene, 25 por pagina).</t>
         </is>
       </c>
     </row>
@@ -2602,11 +2626,19 @@
       </c>
       <c r="N24" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="O24" s="12" t="n"/>
-      <c r="P24" s="12" t="n"/>
+          <t>En revisión</t>
+        </is>
+      </c>
+      <c r="O24" s="12" t="inlineStr">
+        <is>
+          <t>Bryan Chávez</t>
+        </is>
+      </c>
+      <c r="P24" s="12" t="inlineStr">
+        <is>
+          <t>Construida por Bryan Chávez (bloques 231-233). Evidencia S2 con los criterios OK. FALTA la verificacion de los criterios, que es de Catalina.</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="55.15" customHeight="1" s="20">
       <c r="A25" s="13" t="inlineStr">
@@ -3451,11 +3483,17 @@
       </c>
       <c r="H16" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I16" s="11" t="n"/>
-      <c r="J16" s="12" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I16" s="11" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="J16" s="12" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 2, capturas/S2).</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="27.6" customHeight="1" s="20">
       <c r="A17" s="11" t="inlineStr">
@@ -3997,11 +4035,17 @@
       </c>
       <c r="H29" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I29" s="11" t="n"/>
-      <c r="J29" s="12" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I29" s="11" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J29" s="12" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 2, capturas/S2).</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="41.45" customHeight="1" s="20">
       <c r="A30" s="11" t="inlineStr">
@@ -5127,11 +5171,17 @@
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I54" s="11" t="n"/>
-      <c r="J54" s="12" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I54" s="11" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J54" s="12" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 2, capturas/S2).</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="41.45" customHeight="1" s="20">
       <c r="A55" s="11" t="inlineStr">
@@ -6823,11 +6873,17 @@
       </c>
       <c r="H91" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I91" s="11" t="n"/>
-      <c r="J91" s="12" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I91" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J91" s="12" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 2, capturas/S2).</t>
+        </is>
+      </c>
     </row>
     <row r="92" hidden="1" ht="41.45" customHeight="1" s="20">
       <c r="A92" s="11" t="inlineStr">
@@ -7327,11 +7383,17 @@
       </c>
       <c r="H103" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I103" s="11" t="n"/>
-      <c r="J103" s="12" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I103" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J103" s="12" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 2, capturas/S2).</t>
+        </is>
+      </c>
     </row>
     <row r="104" ht="27.6" customHeight="1" s="20">
       <c r="A104" s="11" t="inlineStr">
@@ -8451,11 +8513,17 @@
       </c>
       <c r="H127" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I127" s="11" t="n"/>
-      <c r="J127" s="12" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I127" s="11" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J127" s="12" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 2, capturas/S2).</t>
+        </is>
+      </c>
     </row>
     <row r="128" hidden="1" ht="27.6" customHeight="1" s="20">
       <c r="A128" s="11" t="inlineStr">
@@ -8961,11 +9029,17 @@
       </c>
       <c r="H139" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I139" s="11" t="n"/>
-      <c r="J139" s="12" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I139" s="11" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J139" s="12" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 2, capturas/S2).</t>
+        </is>
+      </c>
     </row>
     <row r="140" ht="41.45" customHeight="1" s="20">
       <c r="A140" s="11" t="inlineStr">
@@ -9429,11 +9503,17 @@
       </c>
       <c r="H149" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I149" s="11" t="n"/>
-      <c r="J149" s="12" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I149" s="11" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J149" s="12" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 2, capturas/S2).</t>
+        </is>
+      </c>
     </row>
     <row r="150" hidden="1" ht="41.45" customHeight="1" s="20">
       <c r="A150" s="11" t="inlineStr">
@@ -9819,11 +9899,17 @@
       </c>
       <c r="H158" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I158" s="11" t="n"/>
-      <c r="J158" s="12" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I158" s="11" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J158" s="12" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 2, capturas/S2).</t>
+        </is>
+      </c>
     </row>
     <row r="159" hidden="1" ht="27.6" customHeight="1" s="20">
       <c r="A159" s="11" t="inlineStr">
@@ -10173,11 +10259,17 @@
       </c>
       <c r="H166" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I166" s="11" t="n"/>
-      <c r="J166" s="12" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I166" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J166" s="12" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 2, capturas/S2).</t>
+        </is>
+      </c>
     </row>
     <row r="167" hidden="1" ht="27.6" customHeight="1" s="20">
       <c r="A167" s="11" t="inlineStr">
@@ -10737,11 +10829,17 @@
       </c>
       <c r="H178" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I178" s="11" t="n"/>
-      <c r="J178" s="12" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I178" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J178" s="12" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 2, capturas/S2).</t>
+        </is>
+      </c>
     </row>
     <row r="179" hidden="1" ht="27.6" customHeight="1" s="20">
       <c r="A179" s="11" t="inlineStr">
@@ -11205,11 +11303,17 @@
       </c>
       <c r="H188" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I188" s="11" t="n"/>
-      <c r="J188" s="12" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I188" s="11" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J188" s="12" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 2, capturas/S2).</t>
+        </is>
+      </c>
     </row>
     <row r="189" hidden="1" ht="27.6" customHeight="1" s="20">
       <c r="A189" s="11" t="inlineStr">
@@ -11709,11 +11813,17 @@
       </c>
       <c r="H200" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I200" s="11" t="n"/>
-      <c r="J200" s="12" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I200" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J200" s="12" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 2, capturas/S2).</t>
+        </is>
+      </c>
     </row>
     <row r="201" ht="41.45" customHeight="1" s="20">
       <c r="A201" s="11" t="inlineStr">
@@ -12645,11 +12755,17 @@
       </c>
       <c r="H220" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I220" s="11" t="n"/>
-      <c r="J220" s="12" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I220" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J220" s="12" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 2, capturas/S2).</t>
+        </is>
+      </c>
     </row>
     <row r="221" hidden="1" ht="27.6" customHeight="1" s="20">
       <c r="A221" s="11" t="inlineStr">
@@ -13149,11 +13265,17 @@
       </c>
       <c r="H232" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I232" s="11" t="n"/>
-      <c r="J232" s="12" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I232" s="11" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J232" s="12" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 2, capturas/S2).</t>
+        </is>
+      </c>
     </row>
     <row r="233" ht="41.45" customHeight="1" s="20">
       <c r="A233" s="11" t="inlineStr">
@@ -13653,11 +13775,17 @@
       </c>
       <c r="H244" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I244" s="11" t="n"/>
-      <c r="J244" s="12" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I244" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J244" s="12" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 2, capturas/S2).</t>
+        </is>
+      </c>
     </row>
     <row r="245" hidden="1" ht="41.45" customHeight="1" s="20">
       <c r="A245" s="11" t="inlineStr">
@@ -14157,11 +14285,17 @@
       </c>
       <c r="H256" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I256" s="11" t="n"/>
-      <c r="J256" s="12" t="n"/>
+          <t>Terminada</t>
+        </is>
+      </c>
+      <c r="I256" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J256" s="12" t="inlineStr">
+        <is>
+          <t>Ejecutadas por Bryan Chávez el 17-09-2026 con evidencia por criterio (Informe de Pruebas Sprint 2, capturas/S2).</t>
+        </is>
+      </c>
     </row>
     <row r="257" ht="41.45" customHeight="1" s="20">
       <c r="A257" s="11" t="inlineStr">
@@ -14409,7 +14543,7 @@
       </c>
       <c r="F6" s="11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -14442,7 +14576,7 @@
       </c>
       <c r="F7" s="13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -14474,7 +14608,7 @@
       </c>
       <c r="F8" s="11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -14506,7 +14640,7 @@
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -14537,7 +14671,7 @@
       </c>
       <c r="F10" s="11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -14570,7 +14704,7 @@
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -14602,7 +14736,7 @@
       </c>
       <c r="F12" s="11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -14729,7 +14863,7 @@
       </c>
       <c r="F16" s="11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -14761,7 +14895,7 @@
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -15116,7 +15250,7 @@
       </c>
       <c r="F28" s="11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -15147,7 +15281,7 @@
       </c>
       <c r="F29" s="13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -15848,7 +15982,7 @@
       </c>
       <c r="F51" s="13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -15880,7 +16014,7 @@
       </c>
       <c r="F52" s="11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -16037,7 +16171,7 @@
       </c>
       <c r="F57" s="13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -16068,7 +16202,7 @@
       </c>
       <c r="F58" s="11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -16099,7 +16233,7 @@
       </c>
       <c r="F59" s="13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -16131,7 +16265,7 @@
       </c>
       <c r="F60" s="11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -16162,7 +16296,7 @@
       </c>
       <c r="F61" s="13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>

</xml_diff>